<commit_message>
updated annotations ted-mdb 1971
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B66A1ED-6C33-4057-934C-ECAF56798245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948351E2-7264-40F3-B29E-3B455860BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="37">
   <si>
     <t>file</t>
   </si>
@@ -127,6 +127,15 @@
   </si>
   <si>
     <t>teddy-744</t>
+  </si>
+  <si>
+    <t>coref</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>discourse</t>
   </si>
 </sst>
 </file>
@@ -462,1353 +471,1447 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.5546875" style="3"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D2" s="3">
         <v>0.67708333333333337</v>
       </c>
-      <c r="D2" s="3">
+      <c r="E2" s="3">
         <v>0.68055555555555558</v>
       </c>
-      <c r="E2" s="3">
-        <f>D2-C2</f>
+      <c r="F2" s="3">
+        <f>E2-D2</f>
         <v>3.4722222222222099E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C3" s="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D3" s="3">
         <v>0.70833333333333337</v>
       </c>
-      <c r="D3" s="3">
+      <c r="E3" s="3">
         <v>0.75</v>
       </c>
-      <c r="E3" s="3">
-        <f t="shared" ref="E3:E66" si="0">D3-C3</f>
+      <c r="F3" s="3">
+        <f t="shared" ref="F3:F66" si="0">E3-D3</f>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C4" s="3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D4" s="3">
         <v>0.55208333333333337</v>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="3">
         <v>0.59375</v>
       </c>
-      <c r="E4" s="3">
+      <c r="F4" s="3">
         <f t="shared" si="0"/>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C5" s="3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D5" s="3">
         <v>0.76041666666666663</v>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="3">
         <v>0.79166666666666663</v>
       </c>
-      <c r="E5" s="3">
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C6" s="3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D6" s="3">
         <v>0.52083333333333337</v>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="3">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
         <v>8.3333333333333259E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="3">
         <v>0.55208333333333337</v>
       </c>
-      <c r="E7" s="3">
-        <f>D7-C7</f>
+      <c r="F7" s="3">
+        <f>E7-D7</f>
         <v>1.0416666666666741E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E8" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E9" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F9" s="3">
-        <f>SUM(E2:E9)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <f>SUM(F2:F9)</f>
         <v>0.21180555555555547</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="3">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="3">
         <v>0.67569444444444449</v>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="3">
         <v>0.72430555555555554</v>
       </c>
-      <c r="E10" s="3">
+      <c r="F10" s="3">
         <f t="shared" si="0"/>
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="3">
         <v>0.56111111111111112</v>
       </c>
-      <c r="D11" s="3">
+      <c r="E11" s="3">
         <v>0.59305555555555556</v>
       </c>
-      <c r="E11" s="3">
-        <f>D11-C11</f>
+      <c r="F11" s="3">
+        <f>E11-D11</f>
         <v>3.1944444444444442E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.77083333333333337</v>
+      </c>
       <c r="E12" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E13" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E14" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+        <v>0.8125</v>
+      </c>
+      <c r="F12" s="3">
+        <f t="shared" si="0"/>
+        <v>4.166666666666663E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F13" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F14" s="3">
-        <f>SUM(E10:E14)</f>
-        <v>8.0555555555555491E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
+        <f>SUM(F10:F14)</f>
+        <v>0.12222222222222212</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="3">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="D15" s="3">
+      <c r="E15" s="3">
         <v>0.59583333333333333</v>
       </c>
-      <c r="E15" s="3">
+      <c r="F15" s="3">
         <f t="shared" si="0"/>
         <v>1.2499999999999956E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C16" s="3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D16" s="3">
         <v>0.25</v>
       </c>
-      <c r="D16" s="3">
+      <c r="E16" s="3">
         <v>0.29166666666666669</v>
       </c>
-      <c r="E16" s="3">
+      <c r="F16" s="3">
         <f t="shared" si="0"/>
         <v>4.1666666666666685E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C17" s="3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D17" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D17" s="3">
+      <c r="E17" s="3">
         <v>0.71180555555555558</v>
       </c>
-      <c r="E17" s="3">
+      <c r="F17" s="3">
         <f t="shared" si="0"/>
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E18" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E19" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E20" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E21" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F18" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F19" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F20" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F21" s="3">
-        <f>SUM(E15:E21)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <f>SUM(F15:F21)</f>
         <v>9.9305555555555591E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E22" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F22" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="3">
+        <v>34</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D23" s="3">
+      <c r="E23" s="3">
         <v>0.68055555555555558</v>
       </c>
-      <c r="E23" s="3">
+      <c r="F23" s="3">
         <f t="shared" si="0"/>
         <v>1.3888888888888951E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C24" s="3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D24" s="3">
         <v>0.72222222222222221</v>
       </c>
-      <c r="D24" s="3">
+      <c r="E24" s="3">
         <v>0.74305555555555558</v>
       </c>
-      <c r="E24" s="3">
+      <c r="F24" s="3">
         <f t="shared" si="0"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C25" s="3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D25" s="3">
         <v>0.5</v>
       </c>
-      <c r="D25" s="3">
+      <c r="E25" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E25" s="3">
+      <c r="F25" s="3">
         <f t="shared" si="0"/>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E26" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E27" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E28" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F26" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F27" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F28" s="3">
-        <f>SUM(E23:E28)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G28" s="3">
+        <f>SUM(F23:F28)</f>
         <v>7.6388888888888951E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="3">
+        <v>34</v>
+      </c>
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="3">
         <v>0.6333333333333333</v>
       </c>
-      <c r="D29" s="3">
+      <c r="E29" s="3">
         <v>0.64930555555555558</v>
       </c>
-      <c r="E29" s="3">
+      <c r="F29" s="3">
         <f t="shared" si="0"/>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C30" s="3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D30" s="3">
         <v>0.4548611111111111</v>
       </c>
-      <c r="D30" s="3">
+      <c r="E30" s="3">
         <v>0.47222222222222221</v>
       </c>
-      <c r="E30" s="3">
+      <c r="F30" s="3">
         <f t="shared" si="0"/>
         <v>1.7361111111111105E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E31" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E32" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E33" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F31" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F32" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F33" s="3">
-        <f>SUM(E29:E32)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <f>SUM(F29:F32)</f>
         <v>3.3333333333333381E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="3">
+        <v>34</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="3">
         <v>0.49652777777777779</v>
       </c>
-      <c r="D34" s="3">
+      <c r="E34" s="3">
         <v>0.51736111111111116</v>
       </c>
-      <c r="E34" s="3">
+      <c r="F34" s="3">
         <f t="shared" si="0"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C35" s="3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D35" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D35" s="3">
+      <c r="E35" s="3">
         <v>0.67847222222222225</v>
       </c>
-      <c r="E35" s="3">
+      <c r="F35" s="3">
         <f t="shared" si="0"/>
         <v>1.1805555555555625E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E36" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E37" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E38" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F36" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F37" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F38" s="3">
-        <f>SUM(E34:E38)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
+        <f>SUM(F34:F38)</f>
         <v>3.2638888888888995E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E39" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F39" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" s="3">
+        <v>34</v>
+      </c>
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="D40" s="3">
+      <c r="E40" s="3">
         <v>0.60069444444444442</v>
       </c>
-      <c r="E40" s="3">
+      <c r="F40" s="3">
         <f t="shared" si="0"/>
         <v>1.7361111111111049E-2</v>
       </c>
-      <c r="F40" s="3"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C41" s="3">
+      <c r="G40" s="3"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="3">
         <v>0.57638888888888884</v>
       </c>
-      <c r="D41" s="3">
+      <c r="E41" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E41" s="3">
+      <c r="F41" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444445308E-3</v>
       </c>
-      <c r="F41" s="3"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E42" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F42" s="3"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E43" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="G41" s="3"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F42" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G42" s="3"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F43" s="3">
-        <f>SUM(E40:E43)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G43" s="3">
+        <f>SUM(F40:F43)</f>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" s="3">
+        <v>34</v>
+      </c>
+      <c r="C44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="3">
         <v>0.79513888888888884</v>
       </c>
-      <c r="D44" s="3">
+      <c r="E44" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="E44" s="3">
+      <c r="F44" s="3">
         <f t="shared" si="0"/>
         <v>1.0416666666666741E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C45" s="3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D45" s="3">
         <v>0.49652777777777779</v>
       </c>
-      <c r="D45" s="3">
+      <c r="E45" s="3">
         <v>0.50694444444444442</v>
       </c>
-      <c r="E45" s="3">
+      <c r="F45" s="3">
         <f t="shared" si="0"/>
         <v>1.041666666666663E-2</v>
       </c>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C46" s="3">
+      <c r="G45" s="3"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D46" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="D46" s="3">
+      <c r="E46" s="3">
         <v>0.59375</v>
       </c>
-      <c r="E46" s="3">
+      <c r="F46" s="3">
         <f t="shared" si="0"/>
         <v>1.041666666666663E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E47" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E48" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F47" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F48" s="3">
-        <f>SUM(E44:E48)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G48" s="3">
+        <f>SUM(F44:F48)</f>
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>16</v>
       </c>
       <c r="B49" t="s">
-        <v>9</v>
-      </c>
-      <c r="C49" s="3">
+        <v>34</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="3">
         <v>0.50347222222222221</v>
       </c>
-      <c r="D49" s="3">
+      <c r="E49" s="3">
         <v>0.52777777777777779</v>
       </c>
-      <c r="E49" s="3">
+      <c r="F49" s="3">
         <f t="shared" si="0"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C50" s="3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D50" s="3">
         <v>0.76388888888888884</v>
       </c>
-      <c r="D50" s="3">
+      <c r="E50" s="3">
         <v>0.77083333333333337</v>
       </c>
-      <c r="E50" s="3">
+      <c r="F50" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444445308E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E51" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F51" s="3">
-        <f>SUM(E49:E51)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G51" s="3">
+        <f>SUM(F49:F51)</f>
         <v>3.1250000000000111E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>17</v>
       </c>
       <c r="B52" t="s">
-        <v>9</v>
-      </c>
-      <c r="C52" s="3">
+        <v>34</v>
+      </c>
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="3">
         <v>0.7729166666666667</v>
       </c>
-      <c r="D52" s="3">
+      <c r="E52" s="3">
         <v>0.79374999999999996</v>
       </c>
-      <c r="E52" s="3">
+      <c r="F52" s="3">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C53" s="3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D53" s="3">
         <v>0.60069444444444442</v>
       </c>
-      <c r="D53" s="3">
+      <c r="E53" s="3">
         <v>0.60763888888888884</v>
       </c>
-      <c r="E53" s="3">
+      <c r="F53" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444444198E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C54" s="3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D54" s="3">
         <v>0.61458333333333337</v>
       </c>
-      <c r="D54" s="3">
+      <c r="E54" s="3">
         <v>0.62847222222222221</v>
       </c>
-      <c r="E54" s="3">
+      <c r="F54" s="3">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E55" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F55" s="3">
-        <f>SUM(E52:E54)</f>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G55" s="3">
+        <f>SUM(F52:F54)</f>
         <v>4.1666666666666519E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>18</v>
       </c>
       <c r="B56" t="s">
-        <v>9</v>
-      </c>
-      <c r="C56" s="3">
+        <v>34</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="D56" s="3">
+      <c r="E56" s="3">
         <v>0.83333333333333337</v>
       </c>
-      <c r="E56" s="3">
+      <c r="F56" s="3">
         <f t="shared" si="0"/>
         <v>2.777777777777779E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C57" s="3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D57" s="3">
         <v>0.68402777777777779</v>
       </c>
-      <c r="D57" s="3">
+      <c r="E57" s="3">
         <v>0.69791666666666663</v>
       </c>
-      <c r="E57" s="3">
+      <c r="F57" s="3">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C58" s="3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D58" s="3">
         <v>0.67847222222222225</v>
       </c>
-      <c r="D58" s="3">
+      <c r="E58" s="3">
         <v>0.69930555555555551</v>
       </c>
-      <c r="E58" s="3">
+      <c r="F58" s="3">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
       </c>
-      <c r="F58" s="3">
-        <f>SUM(E56:E58)</f>
+      <c r="G58" s="3">
+        <f>SUM(F56:F58)</f>
         <v>6.2499999999999889E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E59" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F59" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>9</v>
-      </c>
-      <c r="C60" s="3">
+        <v>34</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" s="3">
         <v>0.71527777777777779</v>
       </c>
-      <c r="D60" s="3">
+      <c r="E60" s="3">
         <v>0.71944444444444444</v>
       </c>
-      <c r="E60" s="3">
+      <c r="F60" s="3">
         <f t="shared" si="0"/>
         <v>4.1666666666666519E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C61" s="3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D61" s="3">
         <v>0.5</v>
       </c>
-      <c r="D61" s="3">
+      <c r="E61" s="3">
         <v>0.52083333333333337</v>
       </c>
-      <c r="E61" s="3">
+      <c r="F61" s="3">
         <f t="shared" si="0"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C62" s="3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D62" s="3">
         <v>0.60763888888888884</v>
       </c>
-      <c r="D62" s="3">
+      <c r="E62" s="3">
         <v>0.625</v>
       </c>
-      <c r="E62" s="3">
+      <c r="F62" s="3">
         <f t="shared" si="0"/>
         <v>1.736111111111116E-2</v>
       </c>
-      <c r="F62" s="3">
-        <f>SUM(E60:E62)</f>
+      <c r="G62" s="3">
+        <f>SUM(F60:F62)</f>
         <v>4.2361111111111183E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E63" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F63" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>20</v>
       </c>
       <c r="B64" t="s">
-        <v>9</v>
-      </c>
-      <c r="C64" s="3">
+        <v>34</v>
+      </c>
+      <c r="C64" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" s="3">
         <v>0.54513888888888884</v>
       </c>
-      <c r="D64" s="3">
+      <c r="E64" s="3">
         <v>0.5625</v>
       </c>
-      <c r="E64" s="3">
+      <c r="F64" s="3">
         <f t="shared" si="0"/>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C65" s="3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D65" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="D65" s="3">
+      <c r="E65" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E65" s="3">
+      <c r="F65" s="3">
         <f t="shared" si="0"/>
         <v>1.0416666666666741E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C66" s="3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D66" s="3">
         <v>0.75555555555555554</v>
       </c>
-      <c r="D66" s="3">
+      <c r="E66" s="3">
         <v>0.75902777777777775</v>
       </c>
-      <c r="E66" s="3">
+      <c r="F66" s="3">
         <f t="shared" si="0"/>
         <v>3.4722222222222099E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E67" s="3">
-        <f t="shared" ref="E67:E122" si="1">D67-C67</f>
-        <v>0</v>
-      </c>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F67" s="3">
-        <f>SUM(E64:E67)</f>
+        <f t="shared" ref="F67:F122" si="1">E67-D67</f>
+        <v>0</v>
+      </c>
+      <c r="G67" s="3">
+        <f>SUM(F64:F67)</f>
         <v>3.1250000000000111E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>21</v>
       </c>
       <c r="B68" t="s">
-        <v>9</v>
-      </c>
-      <c r="C68" s="3">
+        <v>34</v>
+      </c>
+      <c r="C68" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" s="3">
         <v>0.59166666666666667</v>
       </c>
-      <c r="D68" s="3">
+      <c r="E68" s="3">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E68" s="3">
+      <c r="F68" s="3">
         <f t="shared" si="1"/>
         <v>1.2499999999999956E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C69" s="3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D69" s="3">
         <v>0.73263888888888884</v>
       </c>
-      <c r="D69" s="3">
+      <c r="E69" s="3">
         <v>0.75347222222222221</v>
       </c>
-      <c r="E69" s="3">
+      <c r="F69" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E70" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E71" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F70" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F71" s="3">
-        <f>SUM(E68:E71)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G71" s="3">
+        <f>SUM(F68:F71)</f>
         <v>3.3333333333333326E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>22</v>
       </c>
       <c r="B72" t="s">
-        <v>9</v>
-      </c>
-      <c r="C72" s="3">
+        <v>34</v>
+      </c>
+      <c r="C72" t="s">
+        <v>9</v>
+      </c>
+      <c r="D72" s="3">
         <v>0.59305555555555556</v>
       </c>
-      <c r="D72" s="3">
+      <c r="E72" s="3">
         <v>0.61527777777777781</v>
       </c>
-      <c r="E72" s="3">
+      <c r="F72" s="3">
         <f t="shared" si="1"/>
         <v>2.2222222222222254E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E73" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E74" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F73" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F74" s="3">
-        <f>SUM(E72:E74)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G74" s="3">
+        <f>SUM(F72:F74)</f>
         <v>2.2222222222222254E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>23</v>
       </c>
       <c r="B75" t="s">
-        <v>9</v>
-      </c>
-      <c r="C75" s="3">
+        <v>34</v>
+      </c>
+      <c r="C75" t="s">
+        <v>9</v>
+      </c>
+      <c r="D75" s="3">
         <v>0.65625</v>
       </c>
-      <c r="D75" s="3">
+      <c r="E75" s="3">
         <v>0.68263888888888891</v>
       </c>
-      <c r="E75" s="3">
+      <c r="F75" s="3">
         <f t="shared" si="1"/>
         <v>2.6388888888888906E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E76" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E77" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F76" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F77" s="3">
-        <f>SUM(E75:E77)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G77" s="3">
+        <f>SUM(F75:F77)</f>
         <v>2.6388888888888906E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>24</v>
       </c>
       <c r="B78" t="s">
-        <v>9</v>
-      </c>
-      <c r="C78" s="3">
+        <v>34</v>
+      </c>
+      <c r="C78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D78" s="3">
         <v>0.63402777777777775</v>
       </c>
-      <c r="D78" s="3">
+      <c r="E78" s="3">
         <v>0.66319444444444442</v>
       </c>
-      <c r="E78" s="3">
+      <c r="F78" s="3">
         <f t="shared" si="1"/>
         <v>2.9166666666666674E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E79" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E80" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F79" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F80" s="3">
-        <f>SUM(E78:E80)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G80" s="3">
+        <f>SUM(F78:F80)</f>
         <v>2.9166666666666674E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>25</v>
       </c>
       <c r="B81" t="s">
-        <v>9</v>
-      </c>
-      <c r="C81" s="3">
+        <v>34</v>
+      </c>
+      <c r="C81" t="s">
+        <v>9</v>
+      </c>
+      <c r="D81" s="3">
         <v>0.58402777777777781</v>
       </c>
-      <c r="D81" s="3">
+      <c r="E81" s="3">
         <v>0.59791666666666665</v>
       </c>
-      <c r="E81" s="3">
+      <c r="F81" s="3">
         <f t="shared" si="1"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C82" s="3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D82" s="3">
         <v>0.74652777777777779</v>
       </c>
-      <c r="D82" s="3">
+      <c r="E82" s="3">
         <v>0.76458333333333328</v>
       </c>
-      <c r="E82" s="3">
+      <c r="F82" s="3">
         <f t="shared" si="1"/>
         <v>1.8055555555555491E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E83" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F83" s="3">
-        <f>SUM(E81:E83)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G83" s="3">
+        <f>SUM(F81:F83)</f>
         <v>3.1944444444444331E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>26</v>
       </c>
       <c r="B84" t="s">
-        <v>9</v>
-      </c>
-      <c r="C84" s="3">
+        <v>34</v>
+      </c>
+      <c r="C84" t="s">
+        <v>9</v>
+      </c>
+      <c r="D84" s="3">
         <v>0.52430555555555558</v>
       </c>
-      <c r="D84" s="3">
+      <c r="E84" s="3">
         <v>0.54305555555555551</v>
       </c>
-      <c r="E84" s="3">
+      <c r="F84" s="3">
         <f t="shared" si="1"/>
         <v>1.8749999999999933E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C85" s="3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D85" s="3">
         <v>0.54722222222222228</v>
       </c>
-      <c r="D85" s="3">
+      <c r="E85" s="3">
         <v>0.5541666666666667</v>
       </c>
-      <c r="E85" s="3">
+      <c r="F85" s="3">
         <f t="shared" si="1"/>
         <v>6.9444444444444198E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E86" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F86" s="3">
-        <f>SUM(E84:E86)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G86" s="3">
+        <f>SUM(F84:F86)</f>
         <v>2.5694444444444353E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>27</v>
       </c>
       <c r="B87" t="s">
-        <v>9</v>
-      </c>
-      <c r="C87" s="3">
+        <v>34</v>
+      </c>
+      <c r="C87" t="s">
+        <v>9</v>
+      </c>
+      <c r="D87" s="3">
         <v>0.46527777777777779</v>
       </c>
-      <c r="D87" s="3">
+      <c r="E87" s="3">
         <v>0.47569444444444442</v>
       </c>
-      <c r="E87" s="3">
+      <c r="F87" s="3">
         <f t="shared" si="1"/>
         <v>1.041666666666663E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C88" s="3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D88" s="3">
         <v>0.50694444444444442</v>
       </c>
-      <c r="D88" s="3">
+      <c r="E88" s="3">
         <v>0.51249999999999996</v>
       </c>
-      <c r="E88" s="3">
+      <c r="F88" s="3">
         <f t="shared" si="1"/>
         <v>5.5555555555555358E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E89" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F89" s="3">
-        <f>SUM(E87:E89)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G89" s="3">
+        <f>SUM(F87:F89)</f>
         <v>1.5972222222222165E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>29</v>
       </c>
       <c r="B90" t="s">
-        <v>9</v>
-      </c>
-      <c r="C90" s="3">
+        <v>34</v>
+      </c>
+      <c r="C90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D90" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="D90" s="3">
+      <c r="E90" s="3">
         <v>0.55763888888888891</v>
       </c>
-      <c r="E90" s="3">
+      <c r="F90" s="3">
         <f t="shared" si="1"/>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E91" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F91" s="3">
-        <f>SUM(E90:E91)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G91" s="3">
+        <f>SUM(F90:F91)</f>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>28</v>
       </c>
       <c r="B92" t="s">
-        <v>9</v>
-      </c>
-      <c r="C92" s="3">
+        <v>34</v>
+      </c>
+      <c r="C92" t="s">
+        <v>9</v>
+      </c>
+      <c r="D92" s="3">
         <v>0.53472222222222221</v>
       </c>
-      <c r="D92" s="3">
+      <c r="E92" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="E92" s="3">
+      <c r="F92" s="3">
         <f t="shared" si="1"/>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E93" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F93" s="3">
-        <f>SUM(E92:E93)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G93" s="3">
+        <f>SUM(F92:F93)</f>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>30</v>
       </c>
       <c r="B94" t="s">
-        <v>9</v>
-      </c>
-      <c r="C94" s="3">
+        <v>34</v>
+      </c>
+      <c r="C94" t="s">
+        <v>9</v>
+      </c>
+      <c r="D94" s="3">
         <v>0.54652777777777772</v>
       </c>
-      <c r="D94" s="3">
+      <c r="E94" s="3">
         <v>0.56736111111111109</v>
       </c>
-      <c r="E94" s="3">
+      <c r="F94" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E95" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F95" s="3">
-        <f>SUM(E94:E95)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G95" s="3">
+        <f>SUM(F94:F95)</f>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>31</v>
       </c>
       <c r="B96" t="s">
-        <v>9</v>
-      </c>
-      <c r="C96" s="3">
+        <v>34</v>
+      </c>
+      <c r="C96" t="s">
+        <v>9</v>
+      </c>
+      <c r="D96" s="3">
         <v>0.78125</v>
       </c>
-      <c r="D96" s="3">
+      <c r="E96" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="E96" s="3">
+      <c r="F96" s="3">
         <f t="shared" si="1"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E97" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F97" s="3">
-        <f>SUM(E96:E97)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G97" s="3">
+        <f>SUM(F96:F97)</f>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>32</v>
       </c>
       <c r="B98" t="s">
-        <v>9</v>
-      </c>
-      <c r="C98" s="3">
+        <v>34</v>
+      </c>
+      <c r="C98" t="s">
+        <v>9</v>
+      </c>
+      <c r="D98" s="3">
         <v>0.8125</v>
       </c>
-      <c r="D98" s="3">
+      <c r="E98" s="3">
         <v>0.82986111111111116</v>
       </c>
-      <c r="E98" s="3">
+      <c r="F98" s="3">
         <f t="shared" si="1"/>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E99" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F99" s="3">
-        <f>SUM(E98:E99)</f>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G99" s="3">
+        <f>SUM(F98:F99)</f>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>33</v>
       </c>
       <c r="B100" t="s">
-        <v>9</v>
-      </c>
-      <c r="C100" s="3">
+        <v>34</v>
+      </c>
+      <c r="C100" t="s">
+        <v>9</v>
+      </c>
+      <c r="D100" s="3">
         <v>0.59166666666666667</v>
       </c>
-      <c r="D100" s="3">
+      <c r="E100" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E100" s="3">
+      <c r="F100" s="3">
         <f t="shared" si="1"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C101" s="3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D101" s="3">
         <v>0.78888888888888886</v>
       </c>
-      <c r="D101" s="3">
+      <c r="E101" s="3">
         <v>0.83680555555555558</v>
       </c>
-      <c r="E101" s="3">
+      <c r="F101" s="3">
         <f t="shared" si="1"/>
         <v>4.7916666666666718E-2</v>
       </c>
-      <c r="F101" s="3">
-        <f>SUM(E100:E101)</f>
+      <c r="G101" s="3">
+        <f>SUM(F100:F101)</f>
         <v>0.12291666666666667</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E102" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E103" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E104" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E105" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E106" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E107" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E108" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E109" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E110" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E111" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E112" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E113" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E114" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E115" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E116" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E117" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E118" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E119" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E120" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E121" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E122" s="3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F102" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F103" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F104" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F105" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F106" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F107" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F108" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F109" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F110" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F111" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F112" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F113" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F114" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F115" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F116" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F117" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F118" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F119" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F120" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F121" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F122" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated sentence-level annotations ted-mdb
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39366A05-88C3-4395-ABCA-654F48D7B9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E709A9-6B6C-4641-9361-F8EF2CB78E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="15300" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -471,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -529,7 +529,7 @@
         <v>0.75</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F66" si="0">E3-D3</f>
+        <f t="shared" ref="F3:F67" si="0">E3-D3</f>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
@@ -591,79 +591,91 @@
       <c r="C8" t="s">
         <v>9</v>
       </c>
+      <c r="D8" s="3">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.67708333333333337</v>
+      </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.1666666666666741E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D9" s="3">
+        <v>0.75347222222222221</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.78333333333333333</v>
+      </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="3">
-        <f>SUM(F2:F9)</f>
-        <v>0.21180555555555547</v>
+        <v>2.9861111111111116E-2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="F10" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <f>SUM(F2:F10)</f>
+        <v>0.28333333333333333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="3">
         <v>0.67569444444444449</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E11" s="3">
         <v>0.72430555555555554</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F11" s="3">
         <f t="shared" si="0"/>
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D12" s="3">
         <v>0.56111111111111112</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E12" s="3">
         <v>0.59305555555555556</v>
       </c>
-      <c r="F11" s="3">
-        <f>E11-D11</f>
+      <c r="F12" s="3">
+        <f>E12-D12</f>
         <v>3.1944444444444442E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
         <v>36</v>
       </c>
-      <c r="C12" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="3">
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3">
         <v>0.77083333333333337</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E13" s="3">
         <v>0.8125</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F13" s="3">
         <f t="shared" si="0"/>
         <v>4.166666666666663E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F13" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -671,106 +683,102 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G14" s="3">
-        <f>SUM(F10:F14)</f>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F15" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <f>SUM(F11:F15)</f>
         <v>0.12222222222222212</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>10</v>
       </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="3">
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E16" s="3">
         <v>0.59583333333333333</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F16" s="3">
         <f t="shared" si="0"/>
         <v>1.2499999999999956E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D16" s="3">
-        <v>0.25</v>
-      </c>
-      <c r="E16" s="3">
-        <v>0.29166666666666669</v>
-      </c>
-      <c r="F16" s="3">
-        <f t="shared" si="0"/>
-        <v>4.1666666666666685E-2</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D17" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F17" s="3">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666685E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D18" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E18" s="3">
         <v>0.71180555555555558</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F18" s="3">
         <f t="shared" si="0"/>
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="C18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="3">
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="3">
         <v>0.54583333333333328</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E19" s="3">
         <v>0.55555555555555558</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F19" s="3">
         <f t="shared" si="0"/>
         <v>9.7222222222222987E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="3">
-        <v>0.44791666666666669</v>
-      </c>
-      <c r="E19" s="3">
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="F19" s="3">
-        <f t="shared" si="0"/>
-        <v>3.125E-2</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D20" s="3">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="0"/>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D21" s="3">
         <v>0.7680555555555556</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E21" s="3">
         <v>0.79166666666666663</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F21" s="3">
         <f t="shared" si="0"/>
         <v>2.3611111111111027E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F21" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <f>SUM(F15:F21)</f>
-        <v>0.16388888888888892</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -778,68 +786,78 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G22" s="3">
+        <f>SUM(F16:F22)</f>
+        <v>0.16388888888888892</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="F23" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>11</v>
       </c>
-      <c r="B23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="3">
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E24" s="3">
         <v>0.68055555555555558</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F24" s="3">
         <f t="shared" si="0"/>
         <v>1.3888888888888951E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D24" s="3">
-        <v>0.72222222222222221</v>
-      </c>
-      <c r="E24" s="3">
-        <v>0.74305555555555558</v>
-      </c>
-      <c r="F24" s="3">
-        <f t="shared" si="0"/>
-        <v>2.083333333333337E-2</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D25" s="3">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="E25" s="3">
+        <v>0.74305555555555558</v>
+      </c>
+      <c r="F25" s="3">
+        <f t="shared" si="0"/>
+        <v>2.083333333333337E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D26" s="3">
         <v>0.5</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E26" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F26" s="3">
         <f t="shared" si="0"/>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
         <v>36</v>
       </c>
-      <c r="C26" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.90625</v>
+      </c>
+      <c r="E27" s="3">
+        <v>0.95833333333333337</v>
+      </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5.208333333333337E-2</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -847,66 +865,66 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G28" s="3">
-        <f>SUM(F23:F28)</f>
-        <v>7.6388888888888951E-2</v>
-      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="F29" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G29" s="3">
+        <f>SUM(F24:F29)</f>
+        <v>0.12847222222222232</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B29" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="3">
+      <c r="B30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="3">
         <v>0.6333333333333333</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E30" s="3">
         <v>0.64930555555555558</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F30" s="3">
         <f t="shared" si="0"/>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D30" s="3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D31" s="3">
         <v>0.4548611111111111</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E31" s="3">
         <v>0.47222222222222221</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F31" s="3">
         <f t="shared" si="0"/>
         <v>1.7361111111111105E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B31" t="s">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
         <v>36</v>
       </c>
-      <c r="C31" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="3">
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="3">
         <v>0.44236111111111109</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E32" s="3">
         <v>0.45833333333333331</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F32" s="3">
         <f t="shared" si="0"/>
         <v>1.5972222222222221E-2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F32" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
@@ -914,82 +932,78 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G33" s="3">
-        <f>SUM(F29:F32)</f>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F34" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G34" s="3">
+        <f>SUM(F30:F33)</f>
         <v>4.9305555555555602E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>13</v>
       </c>
-      <c r="B34" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="3">
+      <c r="B35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="3">
         <v>0.49652777777777779</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E35" s="3">
         <v>0.51736111111111116</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F35" s="3">
         <f t="shared" si="0"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D35" s="3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D36" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E36" s="3">
         <v>0.67847222222222225</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F36" s="3">
         <f t="shared" si="0"/>
         <v>1.1805555555555625E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B36" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
         <v>36</v>
       </c>
-      <c r="C36" t="s">
-        <v>9</v>
-      </c>
-      <c r="D36" s="3">
+      <c r="C37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" s="3">
         <v>0.56944444444444442</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E37" s="3">
         <v>0.59375</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F37" s="3">
         <f t="shared" si="0"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D37" s="3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D38" s="3">
         <v>0.69166666666666665</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E38" s="3">
         <v>0.72222222222222221</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F38" s="3">
         <f t="shared" si="0"/>
         <v>3.0555555555555558E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F38" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G38" s="3">
-        <f>SUM(F34:F38)</f>
-        <v>8.7500000000000133E-2</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
@@ -997,46 +1011,49 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="G39" s="3">
+        <f>SUM(F35:F39)</f>
+        <v>8.7500000000000133E-2</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+      <c r="F40" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>14</v>
       </c>
-      <c r="B40" t="s">
-        <v>34</v>
-      </c>
-      <c r="C40" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" s="3">
+      <c r="B41" t="s">
+        <v>34</v>
+      </c>
+      <c r="C41" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E41" s="3">
         <v>0.60069444444444442</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F41" s="3">
         <f t="shared" si="0"/>
         <v>1.7361111111111049E-2</v>
       </c>
-      <c r="G40" s="3"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D41" s="3">
+      <c r="G41" s="3"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="3">
         <v>0.57638888888888884</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E42" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F42" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444445308E-3</v>
-      </c>
-      <c r="G41" s="3"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F42" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
       <c r="G42" s="3"/>
     </row>
@@ -1045,61 +1062,62 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G43" s="3">
-        <f>SUM(F40:F43)</f>
+      <c r="G43" s="3"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F44" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G44" s="3">
+        <f>SUM(F41:F44)</f>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>15</v>
       </c>
-      <c r="B44" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" t="s">
-        <v>9</v>
-      </c>
-      <c r="D44" s="3">
+      <c r="B45" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="3">
         <v>0.79513888888888884</v>
       </c>
-      <c r="E44" s="3">
+      <c r="E45" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F45" s="3">
         <f t="shared" si="0"/>
         <v>1.0416666666666741E-2</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D45" s="3">
-        <v>0.49652777777777779</v>
-      </c>
-      <c r="E45" s="3">
-        <v>0.50694444444444442</v>
-      </c>
-      <c r="F45" s="3">
-        <f t="shared" si="0"/>
-        <v>1.041666666666663E-2</v>
-      </c>
-      <c r="G45" s="3"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D46" s="3">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0.50694444444444442</v>
+      </c>
+      <c r="F46" s="3">
+        <f t="shared" si="0"/>
+        <v>1.041666666666663E-2</v>
+      </c>
+      <c r="G46" s="3"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D47" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E47" s="3">
         <v>0.59375</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F47" s="3">
         <f t="shared" si="0"/>
         <v>1.041666666666663E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F47" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -1107,311 +1125,311 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G48" s="3">
-        <f>SUM(F44:F48)</f>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F49" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G49" s="3">
+        <f>SUM(F45:F49)</f>
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
         <v>16</v>
       </c>
-      <c r="B49" t="s">
-        <v>34</v>
-      </c>
-      <c r="C49" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" s="3">
+      <c r="B50" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="3">
         <v>0.50347222222222221</v>
       </c>
-      <c r="E49" s="3">
+      <c r="E50" s="3">
         <v>0.52777777777777779</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F50" s="3">
         <f t="shared" si="0"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D50" s="3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D51" s="3">
         <v>0.76388888888888884</v>
       </c>
-      <c r="E50" s="3">
+      <c r="E51" s="3">
         <v>0.77083333333333337</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F51" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444445308E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F51" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G51" s="3">
-        <f>SUM(F49:F51)</f>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F52" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G52" s="3">
+        <f>SUM(F50:F52)</f>
         <v>3.1250000000000111E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>17</v>
       </c>
-      <c r="B52" t="s">
-        <v>34</v>
-      </c>
-      <c r="C52" t="s">
-        <v>9</v>
-      </c>
-      <c r="D52" s="3">
+      <c r="B53" t="s">
+        <v>34</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" s="3">
         <v>0.7729166666666667</v>
       </c>
-      <c r="E52" s="3">
+      <c r="E53" s="3">
         <v>0.79374999999999996</v>
       </c>
-      <c r="F52" s="3">
+      <c r="F53" s="3">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D53" s="3">
-        <v>0.60069444444444442</v>
-      </c>
-      <c r="E53" s="3">
-        <v>0.60763888888888884</v>
-      </c>
-      <c r="F53" s="3">
-        <f t="shared" si="0"/>
-        <v>6.9444444444444198E-3</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D54" s="3">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="E54" s="3">
+        <v>0.60763888888888884</v>
+      </c>
+      <c r="F54" s="3">
+        <f t="shared" si="0"/>
+        <v>6.9444444444444198E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D55" s="3">
         <v>0.61458333333333337</v>
       </c>
-      <c r="E54" s="3">
+      <c r="E55" s="3">
         <v>0.62847222222222221</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F55" s="3">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F55" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G55" s="3">
-        <f>SUM(F52:F54)</f>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F56" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G56" s="3">
+        <f>SUM(F53:F55)</f>
         <v>4.1666666666666519E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>18</v>
       </c>
-      <c r="B56" t="s">
-        <v>34</v>
-      </c>
-      <c r="C56" t="s">
-        <v>9</v>
-      </c>
-      <c r="D56" s="3">
+      <c r="B57" t="s">
+        <v>34</v>
+      </c>
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="E56" s="3">
+      <c r="E57" s="3">
         <v>0.83333333333333337</v>
       </c>
-      <c r="F56" s="3">
+      <c r="F57" s="3">
         <f t="shared" si="0"/>
         <v>2.777777777777779E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D57" s="3">
-        <v>0.68402777777777779</v>
-      </c>
-      <c r="E57" s="3">
-        <v>0.69791666666666663</v>
-      </c>
-      <c r="F57" s="3">
-        <f t="shared" si="0"/>
-        <v>1.388888888888884E-2</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D58" s="3">
+        <v>0.68402777777777779</v>
+      </c>
+      <c r="E58" s="3">
+        <v>0.69791666666666663</v>
+      </c>
+      <c r="F58" s="3">
+        <f t="shared" si="0"/>
+        <v>1.388888888888884E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D59" s="3">
         <v>0.67847222222222225</v>
       </c>
-      <c r="E58" s="3">
+      <c r="E59" s="3">
         <v>0.69930555555555551</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F59" s="3">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
       </c>
-      <c r="G58" s="3">
-        <f>SUM(F56:F58)</f>
+      <c r="G59" s="3">
+        <f>SUM(F57:F59)</f>
         <v>6.2499999999999889E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F59" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
+      <c r="F60" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>19</v>
       </c>
-      <c r="B60" t="s">
-        <v>34</v>
-      </c>
-      <c r="C60" t="s">
-        <v>9</v>
-      </c>
-      <c r="D60" s="3">
+      <c r="B61" t="s">
+        <v>34</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" s="3">
         <v>0.71527777777777779</v>
       </c>
-      <c r="E60" s="3">
+      <c r="E61" s="3">
         <v>0.71944444444444444</v>
       </c>
-      <c r="F60" s="3">
+      <c r="F61" s="3">
         <f t="shared" si="0"/>
         <v>4.1666666666666519E-3</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D61" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="E61" s="3">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="F61" s="3">
-        <f t="shared" si="0"/>
-        <v>2.083333333333337E-2</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D62" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E62" s="3">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="F62" s="3">
+        <f t="shared" si="0"/>
+        <v>2.083333333333337E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D63" s="3">
         <v>0.60763888888888884</v>
       </c>
-      <c r="E62" s="3">
+      <c r="E63" s="3">
         <v>0.625</v>
       </c>
-      <c r="F62" s="3">
+      <c r="F63" s="3">
         <f t="shared" si="0"/>
         <v>1.736111111111116E-2</v>
       </c>
-      <c r="G62" s="3">
-        <f>SUM(F60:F62)</f>
+      <c r="G63" s="3">
+        <f>SUM(F61:F63)</f>
         <v>4.2361111111111183E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F63" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+      <c r="F64" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>20</v>
       </c>
-      <c r="B64" t="s">
-        <v>34</v>
-      </c>
-      <c r="C64" t="s">
-        <v>9</v>
-      </c>
-      <c r="D64" s="3">
+      <c r="B65" t="s">
+        <v>34</v>
+      </c>
+      <c r="C65" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" s="3">
         <v>0.54513888888888884</v>
       </c>
-      <c r="E64" s="3">
+      <c r="E65" s="3">
         <v>0.5625</v>
       </c>
-      <c r="F64" s="3">
+      <c r="F65" s="3">
         <f t="shared" si="0"/>
         <v>1.736111111111116E-2</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D65" s="3">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="E65" s="3">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="F65" s="3">
-        <f t="shared" si="0"/>
-        <v>1.0416666666666741E-2</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D66" s="3">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="E66" s="3">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F66" s="3">
+        <f t="shared" si="0"/>
+        <v>1.0416666666666741E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D67" s="3">
         <v>0.75555555555555554</v>
       </c>
-      <c r="E66" s="3">
+      <c r="E67" s="3">
         <v>0.75902777777777775</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F67" s="3">
         <f t="shared" si="0"/>
         <v>3.4722222222222099E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F67" s="3">
-        <f t="shared" ref="F67:F122" si="1">E67-D67</f>
-        <v>0</v>
-      </c>
-      <c r="G67" s="3">
-        <f>SUM(F64:F67)</f>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F68" s="3">
+        <f t="shared" ref="F68:F123" si="1">E68-D68</f>
+        <v>0</v>
+      </c>
+      <c r="G68" s="3">
+        <f>SUM(F65:F68)</f>
         <v>3.1250000000000111E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>21</v>
       </c>
-      <c r="B68" t="s">
-        <v>34</v>
-      </c>
-      <c r="C68" t="s">
-        <v>9</v>
-      </c>
-      <c r="D68" s="3">
+      <c r="B69" t="s">
+        <v>34</v>
+      </c>
+      <c r="C69" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" s="3">
         <v>0.59166666666666667</v>
       </c>
-      <c r="E68" s="3">
+      <c r="E69" s="3">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F68" s="3">
+      <c r="F69" s="3">
         <f t="shared" si="1"/>
         <v>1.2499999999999956E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D69" s="3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D70" s="3">
         <v>0.73263888888888884</v>
       </c>
-      <c r="E69" s="3">
+      <c r="E70" s="3">
         <v>0.75347222222222221</v>
       </c>
-      <c r="F69" s="3">
+      <c r="F70" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F70" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -1419,36 +1437,36 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G71" s="3">
-        <f>SUM(F68:F71)</f>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F72" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G72" s="3">
+        <f>SUM(F69:F72)</f>
         <v>3.3333333333333326E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
         <v>22</v>
       </c>
-      <c r="B72" t="s">
-        <v>34</v>
-      </c>
-      <c r="C72" t="s">
-        <v>9</v>
-      </c>
-      <c r="D72" s="3">
+      <c r="B73" t="s">
+        <v>34</v>
+      </c>
+      <c r="C73" t="s">
+        <v>9</v>
+      </c>
+      <c r="D73" s="3">
         <v>0.59305555555555556</v>
       </c>
-      <c r="E72" s="3">
+      <c r="E73" s="3">
         <v>0.61527777777777781</v>
       </c>
-      <c r="F72" s="3">
+      <c r="F73" s="3">
         <f t="shared" si="1"/>
         <v>2.2222222222222254E-2</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F73" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -1456,36 +1474,36 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G74" s="3">
-        <f>SUM(F72:F74)</f>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F75" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <f>SUM(F73:F75)</f>
         <v>2.2222222222222254E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
         <v>23</v>
       </c>
-      <c r="B75" t="s">
-        <v>34</v>
-      </c>
-      <c r="C75" t="s">
-        <v>9</v>
-      </c>
-      <c r="D75" s="3">
+      <c r="B76" t="s">
+        <v>34</v>
+      </c>
+      <c r="C76" t="s">
+        <v>9</v>
+      </c>
+      <c r="D76" s="3">
         <v>0.65625</v>
       </c>
-      <c r="E75" s="3">
+      <c r="E76" s="3">
         <v>0.68263888888888891</v>
       </c>
-      <c r="F75" s="3">
+      <c r="F76" s="3">
         <f t="shared" si="1"/>
         <v>2.6388888888888906E-2</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F76" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
@@ -1493,36 +1511,36 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G77" s="3">
-        <f>SUM(F75:F77)</f>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F78" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G78" s="3">
+        <f>SUM(F76:F78)</f>
         <v>2.6388888888888906E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
         <v>24</v>
       </c>
-      <c r="B78" t="s">
-        <v>34</v>
-      </c>
-      <c r="C78" t="s">
-        <v>9</v>
-      </c>
-      <c r="D78" s="3">
+      <c r="B79" t="s">
+        <v>34</v>
+      </c>
+      <c r="C79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D79" s="3">
         <v>0.63402777777777775</v>
       </c>
-      <c r="E78" s="3">
+      <c r="E79" s="3">
         <v>0.66319444444444442</v>
       </c>
-      <c r="F78" s="3">
+      <c r="F79" s="3">
         <f t="shared" si="1"/>
         <v>2.9166666666666674E-2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F79" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
@@ -1530,336 +1548,336 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G80" s="3">
-        <f>SUM(F78:F80)</f>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F81" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G81" s="3">
+        <f>SUM(F79:F81)</f>
         <v>2.9166666666666674E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
         <v>25</v>
       </c>
-      <c r="B81" t="s">
-        <v>34</v>
-      </c>
-      <c r="C81" t="s">
-        <v>9</v>
-      </c>
-      <c r="D81" s="3">
+      <c r="B82" t="s">
+        <v>34</v>
+      </c>
+      <c r="C82" t="s">
+        <v>9</v>
+      </c>
+      <c r="D82" s="3">
         <v>0.58402777777777781</v>
       </c>
-      <c r="E81" s="3">
+      <c r="E82" s="3">
         <v>0.59791666666666665</v>
       </c>
-      <c r="F81" s="3">
+      <c r="F82" s="3">
         <f t="shared" si="1"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D82" s="3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D83" s="3">
         <v>0.74652777777777779</v>
       </c>
-      <c r="E82" s="3">
+      <c r="E83" s="3">
         <v>0.76458333333333328</v>
       </c>
-      <c r="F82" s="3">
+      <c r="F83" s="3">
         <f t="shared" si="1"/>
         <v>1.8055555555555491E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F83" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G83" s="3">
-        <f>SUM(F81:F83)</f>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F84" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G84" s="3">
+        <f>SUM(F82:F84)</f>
         <v>3.1944444444444331E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
         <v>26</v>
       </c>
-      <c r="B84" t="s">
-        <v>34</v>
-      </c>
-      <c r="C84" t="s">
-        <v>9</v>
-      </c>
-      <c r="D84" s="3">
+      <c r="B85" t="s">
+        <v>34</v>
+      </c>
+      <c r="C85" t="s">
+        <v>9</v>
+      </c>
+      <c r="D85" s="3">
         <v>0.52430555555555558</v>
       </c>
-      <c r="E84" s="3">
+      <c r="E85" s="3">
         <v>0.54305555555555551</v>
       </c>
-      <c r="F84" s="3">
+      <c r="F85" s="3">
         <f t="shared" si="1"/>
         <v>1.8749999999999933E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D85" s="3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D86" s="3">
         <v>0.54722222222222228</v>
       </c>
-      <c r="E85" s="3">
+      <c r="E86" s="3">
         <v>0.5541666666666667</v>
       </c>
-      <c r="F85" s="3">
+      <c r="F86" s="3">
         <f t="shared" si="1"/>
         <v>6.9444444444444198E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F86" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G86" s="3">
-        <f>SUM(F84:F86)</f>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F87" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G87" s="3">
+        <f>SUM(F85:F87)</f>
         <v>2.5694444444444353E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
         <v>27</v>
       </c>
-      <c r="B87" t="s">
-        <v>34</v>
-      </c>
-      <c r="C87" t="s">
-        <v>9</v>
-      </c>
-      <c r="D87" s="3">
+      <c r="B88" t="s">
+        <v>34</v>
+      </c>
+      <c r="C88" t="s">
+        <v>9</v>
+      </c>
+      <c r="D88" s="3">
         <v>0.46527777777777779</v>
       </c>
-      <c r="E87" s="3">
+      <c r="E88" s="3">
         <v>0.47569444444444442</v>
       </c>
-      <c r="F87" s="3">
+      <c r="F88" s="3">
         <f t="shared" si="1"/>
         <v>1.041666666666663E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D88" s="3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D89" s="3">
         <v>0.50694444444444442</v>
       </c>
-      <c r="E88" s="3">
+      <c r="E89" s="3">
         <v>0.51249999999999996</v>
       </c>
-      <c r="F88" s="3">
+      <c r="F89" s="3">
         <f t="shared" si="1"/>
         <v>5.5555555555555358E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F89" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G89" s="3">
-        <f>SUM(F87:F89)</f>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F90" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G90" s="3">
+        <f>SUM(F88:F90)</f>
         <v>1.5972222222222165E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
         <v>29</v>
       </c>
-      <c r="B90" t="s">
-        <v>34</v>
-      </c>
-      <c r="C90" t="s">
-        <v>9</v>
-      </c>
-      <c r="D90" s="3">
+      <c r="B91" t="s">
+        <v>34</v>
+      </c>
+      <c r="C91" t="s">
+        <v>9</v>
+      </c>
+      <c r="D91" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E90" s="3">
+      <c r="E91" s="3">
         <v>0.55763888888888891</v>
       </c>
-      <c r="F90" s="3">
+      <c r="F91" s="3">
         <f t="shared" si="1"/>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F91" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G91" s="3">
-        <f>SUM(F90:F91)</f>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F92" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G92" s="3">
+        <f>SUM(F91:F92)</f>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
         <v>28</v>
       </c>
-      <c r="B92" t="s">
-        <v>34</v>
-      </c>
-      <c r="C92" t="s">
-        <v>9</v>
-      </c>
-      <c r="D92" s="3">
+      <c r="B93" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" t="s">
+        <v>9</v>
+      </c>
+      <c r="D93" s="3">
         <v>0.53472222222222221</v>
       </c>
-      <c r="E92" s="3">
+      <c r="E93" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="F92" s="3">
+      <c r="F93" s="3">
         <f t="shared" si="1"/>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F93" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G93" s="3">
-        <f>SUM(F92:F93)</f>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F94" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G94" s="3">
+        <f>SUM(F93:F94)</f>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
         <v>30</v>
       </c>
-      <c r="B94" t="s">
-        <v>34</v>
-      </c>
-      <c r="C94" t="s">
-        <v>9</v>
-      </c>
-      <c r="D94" s="3">
+      <c r="B95" t="s">
+        <v>34</v>
+      </c>
+      <c r="C95" t="s">
+        <v>9</v>
+      </c>
+      <c r="D95" s="3">
         <v>0.54652777777777772</v>
       </c>
-      <c r="E94" s="3">
+      <c r="E95" s="3">
         <v>0.56736111111111109</v>
       </c>
-      <c r="F94" s="3">
+      <c r="F95" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F95" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G95" s="3">
-        <f>SUM(F94:F95)</f>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F96" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G96" s="3">
+        <f>SUM(F95:F96)</f>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>31</v>
       </c>
-      <c r="B96" t="s">
-        <v>34</v>
-      </c>
-      <c r="C96" t="s">
-        <v>9</v>
-      </c>
-      <c r="D96" s="3">
+      <c r="B97" t="s">
+        <v>34</v>
+      </c>
+      <c r="C97" t="s">
+        <v>9</v>
+      </c>
+      <c r="D97" s="3">
         <v>0.78125</v>
       </c>
-      <c r="E96" s="3">
+      <c r="E97" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F97" s="3">
         <f t="shared" si="1"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F97" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G97" s="3">
-        <f>SUM(F96:F97)</f>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F98" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G98" s="3">
+        <f>SUM(F97:F98)</f>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
         <v>32</v>
       </c>
-      <c r="B98" t="s">
-        <v>34</v>
-      </c>
-      <c r="C98" t="s">
-        <v>9</v>
-      </c>
-      <c r="D98" s="3">
+      <c r="B99" t="s">
+        <v>34</v>
+      </c>
+      <c r="C99" t="s">
+        <v>9</v>
+      </c>
+      <c r="D99" s="3">
         <v>0.8125</v>
       </c>
-      <c r="E98" s="3">
+      <c r="E99" s="3">
         <v>0.82986111111111116</v>
       </c>
-      <c r="F98" s="3">
+      <c r="F99" s="3">
         <f t="shared" si="1"/>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F99" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G99" s="3">
-        <f>SUM(F98:F99)</f>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F100" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G100" s="3">
+        <f>SUM(F99:F100)</f>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
         <v>33</v>
       </c>
-      <c r="B100" t="s">
-        <v>34</v>
-      </c>
-      <c r="C100" t="s">
-        <v>9</v>
-      </c>
-      <c r="D100" s="3">
+      <c r="B101" t="s">
+        <v>34</v>
+      </c>
+      <c r="C101" t="s">
+        <v>9</v>
+      </c>
+      <c r="D101" s="3">
         <v>0.59166666666666667</v>
       </c>
-      <c r="E100" s="3">
+      <c r="E101" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="F100" s="3">
+      <c r="F101" s="3">
         <f t="shared" si="1"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D101" s="3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D102" s="3">
         <v>0.78888888888888886</v>
       </c>
-      <c r="E101" s="3">
+      <c r="E102" s="3">
         <v>0.83680555555555558</v>
       </c>
-      <c r="F101" s="3">
+      <c r="F102" s="3">
         <f t="shared" si="1"/>
         <v>4.7916666666666718E-2</v>
       </c>
-      <c r="G101" s="3">
-        <f>SUM(F100:F101)</f>
+      <c r="G102" s="3">
+        <f>SUM(F101:F102)</f>
         <v>0.12291666666666667</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F102" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
@@ -1978,6 +1996,12 @@
     </row>
     <row r="122" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F122" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F123" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated discourse annotations and directory structure (annotated coref, discourse, both)
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E709A9-6B6C-4641-9361-F8EF2CB78E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D67D5E3C-E848-4E4D-B635-0649365B098F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="15300" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="37">
   <si>
     <t>file</t>
   </si>
@@ -471,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -1391,7 +1392,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F68" s="3">
-        <f t="shared" ref="F68:F123" si="1">E68-D68</f>
+        <f t="shared" ref="F68:F127" si="1">E68-D68</f>
         <v>0</v>
       </c>
       <c r="G68" s="3">
@@ -1710,127 +1711,125 @@
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B92" t="s">
+        <v>36</v>
+      </c>
+      <c r="C92" t="s">
+        <v>9</v>
+      </c>
+      <c r="D92" s="3">
+        <v>0.59513888888888888</v>
+      </c>
+      <c r="E92" s="3">
+        <v>0.61250000000000004</v>
+      </c>
       <c r="F92" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G92" s="3">
-        <f>SUM(F91:F92)</f>
-        <v>1.5972222222222276E-2</v>
+        <v>1.736111111111116E-2</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
+      <c r="F93" s="3"/>
+      <c r="G93" s="3">
+        <f>SUM(F91:F93)</f>
+        <v>3.3333333333333437E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
         <v>28</v>
       </c>
-      <c r="B93" t="s">
-        <v>34</v>
-      </c>
-      <c r="C93" t="s">
-        <v>9</v>
-      </c>
-      <c r="D93" s="3">
+      <c r="B94" t="s">
+        <v>34</v>
+      </c>
+      <c r="C94" t="s">
+        <v>9</v>
+      </c>
+      <c r="D94" s="3">
         <v>0.53472222222222221</v>
       </c>
-      <c r="E93" s="3">
+      <c r="E94" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="F93" s="3">
+      <c r="F94" s="3">
         <f t="shared" si="1"/>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F94" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G94" s="3">
-        <f>SUM(F93:F94)</f>
-        <v>3.819444444444442E-2</v>
-      </c>
-    </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
+      <c r="B95" t="s">
+        <v>36</v>
+      </c>
+      <c r="C95" t="s">
+        <v>9</v>
+      </c>
+      <c r="D95" s="3">
+        <v>0.61597222222222225</v>
+      </c>
+      <c r="E95" s="3">
+        <v>0.62152777777777779</v>
+      </c>
+      <c r="F95" s="3">
+        <f t="shared" si="1"/>
+        <v>5.5555555555555358E-3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D96" s="3">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="E96" s="3">
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="F96" s="3">
+        <f t="shared" si="1"/>
+        <v>1.8055555555555602E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F97" s="3"/>
+      <c r="G97" s="3">
+        <f>SUM(F94:F97)</f>
+        <v>6.1805555555555558E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
         <v>30</v>
       </c>
-      <c r="B95" t="s">
-        <v>34</v>
-      </c>
-      <c r="C95" t="s">
-        <v>9</v>
-      </c>
-      <c r="D95" s="3">
+      <c r="B98" t="s">
+        <v>34</v>
+      </c>
+      <c r="C98" t="s">
+        <v>9</v>
+      </c>
+      <c r="D98" s="3">
         <v>0.54652777777777772</v>
       </c>
-      <c r="E95" s="3">
+      <c r="E98" s="3">
         <v>0.56736111111111109</v>
       </c>
-      <c r="F95" s="3">
+      <c r="F98" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F96" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G96" s="3">
-        <f>SUM(F95:F96)</f>
-        <v>2.083333333333337E-2</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>31</v>
-      </c>
-      <c r="B97" t="s">
-        <v>34</v>
-      </c>
-      <c r="C97" t="s">
-        <v>9</v>
-      </c>
-      <c r="D97" s="3">
-        <v>0.78125</v>
-      </c>
-      <c r="E97" s="3">
-        <v>0.80555555555555558</v>
-      </c>
-      <c r="F97" s="3">
-        <f t="shared" si="1"/>
-        <v>2.430555555555558E-2</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F98" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G98" s="3">
-        <f>SUM(F97:F98)</f>
-        <v>2.430555555555558E-2</v>
-      </c>
-    </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>32</v>
-      </c>
       <c r="B99" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C99" t="s">
         <v>9</v>
       </c>
       <c r="D99" s="3">
-        <v>0.8125</v>
+        <v>0.59513888888888888</v>
       </c>
       <c r="E99" s="3">
-        <v>0.82986111111111116</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="F99" s="3">
         <f t="shared" si="1"/>
-        <v>1.736111111111116E-2</v>
+        <v>9.0277777777777457E-3</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
@@ -1839,13 +1838,13 @@
         <v>0</v>
       </c>
       <c r="G100" s="3">
-        <f>SUM(F99:F100)</f>
-        <v>1.736111111111116E-2</v>
+        <f>SUM(F98:F100)</f>
+        <v>2.9861111111111116E-2</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B101" t="s">
         <v>34</v>
@@ -1854,36 +1853,45 @@
         <v>9</v>
       </c>
       <c r="D101" s="3">
-        <v>0.59166666666666667</v>
+        <v>0.78125</v>
       </c>
       <c r="E101" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.80555555555555558</v>
       </c>
       <c r="F101" s="3">
         <f t="shared" si="1"/>
-        <v>7.4999999999999956E-2</v>
+        <v>2.430555555555558E-2</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D102" s="3">
-        <v>0.78888888888888886</v>
-      </c>
-      <c r="E102" s="3">
-        <v>0.83680555555555558</v>
-      </c>
       <c r="F102" s="3">
         <f t="shared" si="1"/>
-        <v>4.7916666666666718E-2</v>
+        <v>0</v>
       </c>
       <c r="G102" s="3">
         <f>SUM(F101:F102)</f>
-        <v>0.12291666666666667</v>
+        <v>2.430555555555558E-2</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>32</v>
+      </c>
+      <c r="B103" t="s">
+        <v>34</v>
+      </c>
+      <c r="C103" t="s">
+        <v>9</v>
+      </c>
+      <c r="D103" s="3">
+        <v>0.8125</v>
+      </c>
+      <c r="E103" s="3">
+        <v>0.82986111111111116</v>
+      </c>
       <c r="F103" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.736111111111116E-2</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.3">
@@ -1891,17 +1899,46 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="G104" s="3">
+        <f>SUM(F103:F104)</f>
+        <v>1.736111111111116E-2</v>
+      </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>33</v>
+      </c>
+      <c r="B105" t="s">
+        <v>34</v>
+      </c>
+      <c r="C105" t="s">
+        <v>9</v>
+      </c>
+      <c r="D105" s="3">
+        <v>0.59166666666666667</v>
+      </c>
+      <c r="E105" s="3">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F105" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7.4999999999999956E-2</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D106" s="3">
+        <v>0.78888888888888886</v>
+      </c>
+      <c r="E106" s="3">
+        <v>0.83680555555555558</v>
+      </c>
       <c r="F106" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.7916666666666718E-2</v>
+      </c>
+      <c r="G106" s="3">
+        <f>SUM(F105:F106)</f>
+        <v>0.12291666666666667</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
@@ -2002,6 +2039,30 @@
     </row>
     <row r="123" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F123" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F124" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F125" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F126" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F127" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated discourse annotations (news)
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D67D5E3C-E848-4E4D-B635-0649365B098F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D436C516-A13C-4299-8A84-A93121758224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15480" yWindow="0" windowWidth="7656" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="37">
   <si>
     <t>file</t>
   </si>
@@ -472,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -530,7 +529,7 @@
         <v>0.75</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F67" si="0">E3-D3</f>
+        <f t="shared" ref="F3:F70" si="0">E3-D3</f>
         <v>4.166666666666663E-2</v>
       </c>
     </row>
@@ -1046,6 +1045,12 @@
       <c r="G41" s="3"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
       <c r="D42" s="3">
         <v>0.57638888888888884</v>
       </c>
@@ -1059,415 +1064,427 @@
       <c r="G42" s="3"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="3">
+        <v>0.55902777777777779</v>
+      </c>
+      <c r="E43" s="3">
+        <v>0.56597222222222221</v>
+      </c>
       <c r="F43" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.9444444444444198E-3</v>
       </c>
       <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F44" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G44" s="3">
-        <f>SUM(F41:F44)</f>
-        <v>2.430555555555558E-2</v>
-      </c>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+      <c r="F45" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="3">
+        <f>SUM(F41:F45)</f>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
         <v>15</v>
       </c>
-      <c r="B45" t="s">
-        <v>34</v>
-      </c>
-      <c r="C45" t="s">
-        <v>9</v>
-      </c>
-      <c r="D45" s="3">
+      <c r="B46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="3">
         <v>0.79513888888888884</v>
       </c>
-      <c r="E45" s="3">
+      <c r="E46" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F46" s="3">
         <f t="shared" si="0"/>
         <v>1.0416666666666741E-2</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D46" s="3">
-        <v>0.49652777777777779</v>
-      </c>
-      <c r="E46" s="3">
-        <v>0.50694444444444442</v>
-      </c>
-      <c r="F46" s="3">
-        <f t="shared" si="0"/>
-        <v>1.041666666666663E-2</v>
-      </c>
-      <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D47" s="3">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="E47" s="3">
+        <v>0.50694444444444442</v>
+      </c>
+      <c r="F47" s="3">
+        <f t="shared" si="0"/>
+        <v>1.041666666666663E-2</v>
+      </c>
+      <c r="G47" s="3"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D48" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E47" s="3">
+      <c r="E48" s="3">
         <v>0.59375</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F48" s="3">
         <f t="shared" si="0"/>
         <v>1.041666666666663E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F48" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="3">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="E49" s="3">
+        <v>0.58472222222222225</v>
+      </c>
       <c r="F49" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="3">
-        <f>SUM(F45:F49)</f>
-        <v>3.125E-2</v>
+        <v>1.5277777777777835E-2</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+      <c r="F50" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="3">
+        <f>SUM(F46:F50)</f>
+        <v>4.6527777777777835E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>16</v>
       </c>
-      <c r="B50" t="s">
-        <v>34</v>
-      </c>
-      <c r="C50" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" s="3">
+      <c r="B51" t="s">
+        <v>34</v>
+      </c>
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="3">
         <v>0.50347222222222221</v>
       </c>
-      <c r="E50" s="3">
+      <c r="E51" s="3">
         <v>0.52777777777777779</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F51" s="3">
         <f t="shared" si="0"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D51" s="3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D52" s="3">
         <v>0.76388888888888884</v>
       </c>
-      <c r="E51" s="3">
+      <c r="E52" s="3">
         <v>0.77083333333333337</v>
       </c>
-      <c r="F51" s="3">
+      <c r="F52" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444445308E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F52" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G52" s="3">
-        <f>SUM(F50:F52)</f>
-        <v>3.1250000000000111E-2</v>
-      </c>
-    </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+      <c r="B53" t="s">
+        <v>36</v>
+      </c>
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" s="3">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="E53" s="3">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="F53" s="3">
+        <f t="shared" si="0"/>
+        <v>1.388888888888884E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F54" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="3">
+        <f>SUM(F51:F54)</f>
+        <v>4.5138888888888951E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>17</v>
       </c>
-      <c r="B53" t="s">
-        <v>34</v>
-      </c>
-      <c r="C53" t="s">
-        <v>9</v>
-      </c>
-      <c r="D53" s="3">
+      <c r="B55" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" s="3">
         <v>0.7729166666666667</v>
       </c>
-      <c r="E53" s="3">
+      <c r="E55" s="3">
         <v>0.79374999999999996</v>
       </c>
-      <c r="F53" s="3">
+      <c r="F55" s="3">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D54" s="3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D56" s="3">
         <v>0.60069444444444442</v>
       </c>
-      <c r="E54" s="3">
+      <c r="E56" s="3">
         <v>0.60763888888888884</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F56" s="3">
         <f t="shared" si="0"/>
         <v>6.9444444444444198E-3</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D55" s="3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D57" s="3">
         <v>0.61458333333333337</v>
       </c>
-      <c r="E55" s="3">
+      <c r="E57" s="3">
         <v>0.62847222222222221</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F57" s="3">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F56" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G56" s="3">
-        <f>SUM(F53:F55)</f>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
+        <v>36</v>
+      </c>
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" s="3"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F59" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G59" s="3">
+        <f>SUM(F55:F57)</f>
         <v>4.1666666666666519E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>18</v>
       </c>
-      <c r="B57" t="s">
-        <v>34</v>
-      </c>
-      <c r="C57" t="s">
-        <v>9</v>
-      </c>
-      <c r="D57" s="3">
+      <c r="B60" t="s">
+        <v>34</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="E57" s="3">
+      <c r="E60" s="3">
         <v>0.83333333333333337</v>
       </c>
-      <c r="F57" s="3">
+      <c r="F60" s="3">
         <f t="shared" si="0"/>
         <v>2.777777777777779E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D58" s="3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D61" s="3">
         <v>0.68402777777777779</v>
       </c>
-      <c r="E58" s="3">
+      <c r="E61" s="3">
         <v>0.69791666666666663</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F61" s="3">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D59" s="3">
-        <v>0.67847222222222225</v>
-      </c>
-      <c r="E59" s="3">
-        <v>0.69930555555555551</v>
-      </c>
-      <c r="F59" s="3">
-        <f t="shared" si="0"/>
-        <v>2.0833333333333259E-2</v>
-      </c>
-      <c r="G59" s="3">
-        <f>SUM(F57:F59)</f>
-        <v>6.2499999999999889E-2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F60" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>19</v>
-      </c>
-      <c r="B61" t="s">
-        <v>34</v>
-      </c>
-      <c r="C61" t="s">
-        <v>9</v>
-      </c>
-      <c r="D61" s="3">
-        <v>0.71527777777777779</v>
-      </c>
-      <c r="E61" s="3">
-        <v>0.71944444444444444</v>
-      </c>
-      <c r="F61" s="3">
-        <f t="shared" si="0"/>
-        <v>4.1666666666666519E-3</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D62" s="3">
+        <v>0.67847222222222225</v>
+      </c>
+      <c r="E62" s="3">
+        <v>0.69930555555555551</v>
+      </c>
+      <c r="F62" s="3">
+        <f t="shared" si="0"/>
+        <v>2.0833333333333259E-2</v>
+      </c>
+      <c r="G62" s="3">
+        <f>SUM(F60:F62)</f>
+        <v>6.2499999999999889E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F63" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" t="s">
+        <v>34</v>
+      </c>
+      <c r="C64" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" s="3">
+        <v>0.71527777777777779</v>
+      </c>
+      <c r="E64" s="3">
+        <v>0.71944444444444444</v>
+      </c>
+      <c r="F64" s="3">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666519E-3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D65" s="3">
         <v>0.5</v>
       </c>
-      <c r="E62" s="3">
+      <c r="E65" s="3">
         <v>0.52083333333333337</v>
       </c>
-      <c r="F62" s="3">
+      <c r="F65" s="3">
         <f t="shared" si="0"/>
         <v>2.083333333333337E-2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D63" s="3">
-        <v>0.60763888888888884</v>
-      </c>
-      <c r="E63" s="3">
-        <v>0.625</v>
-      </c>
-      <c r="F63" s="3">
-        <f t="shared" si="0"/>
-        <v>1.736111111111116E-2</v>
-      </c>
-      <c r="G63" s="3">
-        <f>SUM(F61:F63)</f>
-        <v>4.2361111111111183E-2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F64" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>20</v>
-      </c>
-      <c r="B65" t="s">
-        <v>34</v>
-      </c>
-      <c r="C65" t="s">
-        <v>9</v>
-      </c>
-      <c r="D65" s="3">
-        <v>0.54513888888888884</v>
-      </c>
-      <c r="E65" s="3">
-        <v>0.5625</v>
-      </c>
-      <c r="F65" s="3">
-        <f t="shared" si="0"/>
-        <v>1.736111111111116E-2</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D66" s="3">
+        <v>0.60763888888888884</v>
+      </c>
+      <c r="E66" s="3">
+        <v>0.625</v>
+      </c>
+      <c r="F66" s="3">
+        <f t="shared" si="0"/>
+        <v>1.736111111111116E-2</v>
+      </c>
+      <c r="G66" s="3">
+        <f>SUM(F64:F66)</f>
+        <v>4.2361111111111183E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F67" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" t="s">
+        <v>34</v>
+      </c>
+      <c r="C68" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" s="3">
+        <v>0.54513888888888884</v>
+      </c>
+      <c r="E68" s="3">
+        <v>0.5625</v>
+      </c>
+      <c r="F68" s="3">
+        <f t="shared" si="0"/>
+        <v>1.736111111111116E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D69" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="E66" s="3">
+      <c r="E69" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F69" s="3">
         <f t="shared" si="0"/>
         <v>1.0416666666666741E-2</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D67" s="3">
-        <v>0.75555555555555554</v>
-      </c>
-      <c r="E67" s="3">
-        <v>0.75902777777777775</v>
-      </c>
-      <c r="F67" s="3">
-        <f t="shared" si="0"/>
-        <v>3.4722222222222099E-3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F68" s="3">
-        <f t="shared" ref="F68:F127" si="1">E68-D68</f>
-        <v>0</v>
-      </c>
-      <c r="G68" s="3">
-        <f>SUM(F65:F68)</f>
-        <v>3.1250000000000111E-2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>21</v>
-      </c>
-      <c r="B69" t="s">
-        <v>34</v>
-      </c>
-      <c r="C69" t="s">
-        <v>9</v>
-      </c>
-      <c r="D69" s="3">
-        <v>0.59166666666666667</v>
-      </c>
-      <c r="E69" s="3">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="F69" s="3">
-        <f t="shared" si="1"/>
-        <v>1.2499999999999956E-2</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D70" s="3">
-        <v>0.73263888888888884</v>
+        <v>0.75555555555555554</v>
       </c>
       <c r="E70" s="3">
-        <v>0.75347222222222221</v>
+        <v>0.75902777777777775</v>
       </c>
       <c r="F70" s="3">
-        <f t="shared" si="1"/>
-        <v>2.083333333333337E-2</v>
+        <f t="shared" si="0"/>
+        <v>3.4722222222222099E-3</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F71" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="F71:F130" si="1">E71-D71</f>
+        <v>0</v>
+      </c>
+      <c r="G71" s="3">
+        <f>SUM(F68:F71)</f>
+        <v>3.1250000000000111E-2</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>21</v>
+      </c>
+      <c r="B72" t="s">
+        <v>34</v>
+      </c>
+      <c r="C72" t="s">
+        <v>9</v>
+      </c>
+      <c r="D72" s="3">
+        <v>0.59166666666666667</v>
+      </c>
+      <c r="E72" s="3">
+        <v>0.60416666666666663</v>
+      </c>
       <c r="F72" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G72" s="3">
-        <f>SUM(F69:F72)</f>
-        <v>3.3333333333333326E-2</v>
+        <v>1.2499999999999956E-2</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>22</v>
-      </c>
-      <c r="B73" t="s">
-        <v>34</v>
-      </c>
-      <c r="C73" t="s">
-        <v>9</v>
-      </c>
       <c r="D73" s="3">
-        <v>0.59305555555555556</v>
+        <v>0.73263888888888884</v>
       </c>
       <c r="E73" s="3">
-        <v>0.61527777777777781</v>
+        <v>0.75347222222222221</v>
       </c>
       <c r="F73" s="3">
         <f t="shared" si="1"/>
-        <v>2.2222222222222254E-2</v>
+        <v>2.083333333333337E-2</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -1482,13 +1499,13 @@
         <v>0</v>
       </c>
       <c r="G75" s="3">
-        <f>SUM(F73:F75)</f>
-        <v>2.2222222222222254E-2</v>
+        <f>SUM(F72:F75)</f>
+        <v>3.3333333333333326E-2</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B76" t="s">
         <v>34</v>
@@ -1497,14 +1514,14 @@
         <v>9</v>
       </c>
       <c r="D76" s="3">
-        <v>0.65625</v>
+        <v>0.59305555555555556</v>
       </c>
       <c r="E76" s="3">
-        <v>0.68263888888888891</v>
+        <v>0.61527777777777781</v>
       </c>
       <c r="F76" s="3">
         <f t="shared" si="1"/>
-        <v>2.6388888888888906E-2</v>
+        <v>2.2222222222222254E-2</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
@@ -1520,12 +1537,12 @@
       </c>
       <c r="G78" s="3">
         <f>SUM(F76:F78)</f>
-        <v>2.6388888888888906E-2</v>
+        <v>2.2222222222222254E-2</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B79" t="s">
         <v>34</v>
@@ -1534,14 +1551,14 @@
         <v>9</v>
       </c>
       <c r="D79" s="3">
-        <v>0.63402777777777775</v>
+        <v>0.65625</v>
       </c>
       <c r="E79" s="3">
-        <v>0.66319444444444442</v>
+        <v>0.68263888888888891</v>
       </c>
       <c r="F79" s="3">
         <f t="shared" si="1"/>
-        <v>2.9166666666666674E-2</v>
+        <v>2.6388888888888906E-2</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
@@ -1557,12 +1574,12 @@
       </c>
       <c r="G81" s="3">
         <f>SUM(F79:F81)</f>
-        <v>2.9166666666666674E-2</v>
+        <v>2.6388888888888906E-2</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B82" t="s">
         <v>34</v>
@@ -1571,26 +1588,20 @@
         <v>9</v>
       </c>
       <c r="D82" s="3">
-        <v>0.58402777777777781</v>
+        <v>0.63402777777777775</v>
       </c>
       <c r="E82" s="3">
-        <v>0.59791666666666665</v>
+        <v>0.66319444444444442</v>
       </c>
       <c r="F82" s="3">
         <f t="shared" si="1"/>
-        <v>1.388888888888884E-2</v>
+        <v>2.9166666666666674E-2</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D83" s="3">
-        <v>0.74652777777777779</v>
-      </c>
-      <c r="E83" s="3">
-        <v>0.76458333333333328</v>
-      </c>
       <c r="F83" s="3">
         <f t="shared" si="1"/>
-        <v>1.8055555555555491E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
@@ -1600,12 +1611,12 @@
       </c>
       <c r="G84" s="3">
         <f>SUM(F82:F84)</f>
-        <v>3.1944444444444331E-2</v>
+        <v>2.9166666666666674E-2</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B85" t="s">
         <v>34</v>
@@ -1614,26 +1625,26 @@
         <v>9</v>
       </c>
       <c r="D85" s="3">
-        <v>0.52430555555555558</v>
+        <v>0.58402777777777781</v>
       </c>
       <c r="E85" s="3">
-        <v>0.54305555555555551</v>
+        <v>0.59791666666666665</v>
       </c>
       <c r="F85" s="3">
         <f t="shared" si="1"/>
-        <v>1.8749999999999933E-2</v>
+        <v>1.388888888888884E-2</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D86" s="3">
-        <v>0.54722222222222228</v>
+        <v>0.74652777777777779</v>
       </c>
       <c r="E86" s="3">
-        <v>0.5541666666666667</v>
+        <v>0.76458333333333328</v>
       </c>
       <c r="F86" s="3">
         <f t="shared" si="1"/>
-        <v>6.9444444444444198E-3</v>
+        <v>1.8055555555555491E-2</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
@@ -1643,12 +1654,12 @@
       </c>
       <c r="G87" s="3">
         <f>SUM(F85:F87)</f>
-        <v>2.5694444444444353E-2</v>
+        <v>3.1944444444444331E-2</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B88" t="s">
         <v>34</v>
@@ -1657,26 +1668,26 @@
         <v>9</v>
       </c>
       <c r="D88" s="3">
-        <v>0.46527777777777779</v>
+        <v>0.52430555555555558</v>
       </c>
       <c r="E88" s="3">
-        <v>0.47569444444444442</v>
+        <v>0.54305555555555551</v>
       </c>
       <c r="F88" s="3">
         <f t="shared" si="1"/>
-        <v>1.041666666666663E-2</v>
+        <v>1.8749999999999933E-2</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D89" s="3">
-        <v>0.50694444444444442</v>
+        <v>0.54722222222222228</v>
       </c>
       <c r="E89" s="3">
-        <v>0.51249999999999996</v>
+        <v>0.5541666666666667</v>
       </c>
       <c r="F89" s="3">
         <f t="shared" si="1"/>
-        <v>5.5555555555555358E-3</v>
+        <v>6.9444444444444198E-3</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
@@ -1686,12 +1697,12 @@
       </c>
       <c r="G90" s="3">
         <f>SUM(F88:F90)</f>
-        <v>1.5972222222222165E-2</v>
+        <v>2.5694444444444353E-2</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B91" t="s">
         <v>34</v>
@@ -1700,44 +1711,41 @@
         <v>9</v>
       </c>
       <c r="D91" s="3">
-        <v>0.54166666666666663</v>
+        <v>0.46527777777777779</v>
       </c>
       <c r="E91" s="3">
-        <v>0.55763888888888891</v>
+        <v>0.47569444444444442</v>
       </c>
       <c r="F91" s="3">
         <f t="shared" si="1"/>
-        <v>1.5972222222222276E-2</v>
+        <v>1.041666666666663E-2</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B92" t="s">
-        <v>36</v>
-      </c>
-      <c r="C92" t="s">
-        <v>9</v>
-      </c>
       <c r="D92" s="3">
-        <v>0.59513888888888888</v>
+        <v>0.50694444444444442</v>
       </c>
       <c r="E92" s="3">
-        <v>0.61250000000000004</v>
+        <v>0.51249999999999996</v>
       </c>
       <c r="F92" s="3">
         <f t="shared" si="1"/>
-        <v>1.736111111111116E-2</v>
+        <v>5.5555555555555358E-3</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F93" s="3"/>
+      <c r="F93" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="G93" s="3">
         <f>SUM(F91:F93)</f>
-        <v>3.3333333333333437E-2</v>
+        <v>1.5972222222222165E-2</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B94" t="s">
         <v>34</v>
@@ -1746,14 +1754,14 @@
         <v>9</v>
       </c>
       <c r="D94" s="3">
-        <v>0.53472222222222221</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="E94" s="3">
-        <v>0.57291666666666663</v>
+        <v>0.55763888888888891</v>
       </c>
       <c r="F94" s="3">
         <f t="shared" si="1"/>
-        <v>3.819444444444442E-2</v>
+        <v>1.5972222222222276E-2</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
@@ -1764,181 +1772,180 @@
         <v>9</v>
       </c>
       <c r="D95" s="3">
+        <v>0.59513888888888888</v>
+      </c>
+      <c r="E95" s="3">
+        <v>0.61250000000000004</v>
+      </c>
+      <c r="F95" s="3">
+        <f t="shared" si="1"/>
+        <v>1.736111111111116E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F96" s="3"/>
+      <c r="G96" s="3">
+        <f>SUM(F94:F96)</f>
+        <v>3.3333333333333437E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>28</v>
+      </c>
+      <c r="B97" t="s">
+        <v>34</v>
+      </c>
+      <c r="C97" t="s">
+        <v>9</v>
+      </c>
+      <c r="D97" s="3">
+        <v>0.53472222222222221</v>
+      </c>
+      <c r="E97" s="3">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="F97" s="3">
+        <f t="shared" si="1"/>
+        <v>3.819444444444442E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
+        <v>36</v>
+      </c>
+      <c r="C98" t="s">
+        <v>9</v>
+      </c>
+      <c r="D98" s="3">
         <v>0.61597222222222225</v>
       </c>
-      <c r="E95" s="3">
+      <c r="E98" s="3">
         <v>0.62152777777777779</v>
       </c>
-      <c r="F95" s="3">
+      <c r="F98" s="3">
         <f t="shared" si="1"/>
         <v>5.5555555555555358E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D96" s="3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D99" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="E96" s="3">
+      <c r="E99" s="3">
         <v>0.59097222222222223</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F99" s="3">
         <f t="shared" si="1"/>
         <v>1.8055555555555602E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F97" s="3"/>
-      <c r="G97" s="3">
-        <f>SUM(F94:F97)</f>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F100" s="3"/>
+      <c r="G100" s="3">
+        <f>SUM(F97:F100)</f>
         <v>6.1805555555555558E-2</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>30</v>
-      </c>
-      <c r="B98" t="s">
-        <v>34</v>
-      </c>
-      <c r="C98" t="s">
-        <v>9</v>
-      </c>
-      <c r="D98" s="3">
-        <v>0.54652777777777772</v>
-      </c>
-      <c r="E98" s="3">
-        <v>0.56736111111111109</v>
-      </c>
-      <c r="F98" s="3">
-        <f t="shared" si="1"/>
-        <v>2.083333333333337E-2</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B99" t="s">
-        <v>36</v>
-      </c>
-      <c r="C99" t="s">
-        <v>9</v>
-      </c>
-      <c r="D99" s="3">
-        <v>0.59513888888888888</v>
-      </c>
-      <c r="E99" s="3">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="F99" s="3">
-        <f t="shared" si="1"/>
-        <v>9.0277777777777457E-3</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F100" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G100" s="3">
-        <f>SUM(F98:F100)</f>
-        <v>2.9861111111111116E-2</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
+        <v>30</v>
+      </c>
+      <c r="B101" t="s">
+        <v>34</v>
+      </c>
+      <c r="C101" t="s">
+        <v>9</v>
+      </c>
+      <c r="D101" s="3">
+        <v>0.54652777777777772</v>
+      </c>
+      <c r="E101" s="3">
+        <v>0.56736111111111109</v>
+      </c>
+      <c r="F101" s="3">
+        <f t="shared" si="1"/>
+        <v>2.083333333333337E-2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B102" t="s">
+        <v>36</v>
+      </c>
+      <c r="C102" t="s">
+        <v>9</v>
+      </c>
+      <c r="D102" s="3">
+        <v>0.59513888888888888</v>
+      </c>
+      <c r="E102" s="3">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F102" s="3">
+        <f t="shared" si="1"/>
+        <v>9.0277777777777457E-3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F103" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G103" s="3">
+        <f>SUM(F101:F103)</f>
+        <v>2.9861111111111116E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
         <v>31</v>
       </c>
-      <c r="B101" t="s">
-        <v>34</v>
-      </c>
-      <c r="C101" t="s">
-        <v>9</v>
-      </c>
-      <c r="D101" s="3">
+      <c r="B104" t="s">
+        <v>34</v>
+      </c>
+      <c r="C104" t="s">
+        <v>9</v>
+      </c>
+      <c r="D104" s="3">
         <v>0.78125</v>
       </c>
-      <c r="E101" s="3">
+      <c r="E104" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="F101" s="3">
+      <c r="F104" s="3">
         <f t="shared" si="1"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F102" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G102" s="3">
-        <f>SUM(F101:F102)</f>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F105" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G105" s="3">
+        <f>SUM(F104:F105)</f>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
         <v>32</v>
       </c>
-      <c r="B103" t="s">
-        <v>34</v>
-      </c>
-      <c r="C103" t="s">
-        <v>9</v>
-      </c>
-      <c r="D103" s="3">
+      <c r="B106" t="s">
+        <v>34</v>
+      </c>
+      <c r="C106" t="s">
+        <v>9</v>
+      </c>
+      <c r="D106" s="3">
         <v>0.8125</v>
       </c>
-      <c r="E103" s="3">
+      <c r="E106" s="3">
         <v>0.82986111111111116</v>
       </c>
-      <c r="F103" s="3">
+      <c r="F106" s="3">
         <f t="shared" si="1"/>
         <v>1.736111111111116E-2</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F104" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G104" s="3">
-        <f>SUM(F103:F104)</f>
-        <v>1.736111111111116E-2</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>33</v>
-      </c>
-      <c r="B105" t="s">
-        <v>34</v>
-      </c>
-      <c r="C105" t="s">
-        <v>9</v>
-      </c>
-      <c r="D105" s="3">
-        <v>0.59166666666666667</v>
-      </c>
-      <c r="E105" s="3">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F105" s="3">
-        <f t="shared" si="1"/>
-        <v>7.4999999999999956E-2</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D106" s="3">
-        <v>0.78888888888888886</v>
-      </c>
-      <c r="E106" s="3">
-        <v>0.83680555555555558</v>
-      </c>
-      <c r="F106" s="3">
-        <f t="shared" si="1"/>
-        <v>4.7916666666666718E-2</v>
-      </c>
-      <c r="G106" s="3">
-        <f>SUM(F105:F106)</f>
-        <v>0.12291666666666667</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
@@ -1946,17 +1953,46 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="G107" s="3">
+        <f>SUM(F106:F107)</f>
+        <v>1.736111111111116E-2</v>
+      </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>33</v>
+      </c>
+      <c r="B108" t="s">
+        <v>34</v>
+      </c>
+      <c r="C108" t="s">
+        <v>9</v>
+      </c>
+      <c r="D108" s="3">
+        <v>0.59166666666666667</v>
+      </c>
+      <c r="E108" s="3">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F108" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7.4999999999999956E-2</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D109" s="3">
+        <v>0.78888888888888886</v>
+      </c>
+      <c r="E109" s="3">
+        <v>0.83680555555555558</v>
+      </c>
       <c r="F109" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.7916666666666718E-2</v>
+      </c>
+      <c r="G109" s="3">
+        <f>SUM(F108:F109)</f>
+        <v>0.12291666666666667</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.3">
@@ -2063,6 +2099,24 @@
     </row>
     <row r="127" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F127" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F128" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F129" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F130" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
discourse annotations for cnn.167026.xlsx
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB686A2-4895-4469-B03A-0BAE1559476F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B27D7DF-EC65-47B1-8A4F-F1B18EBB4659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5400" yWindow="1776" windowWidth="13080" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16380" yWindow="0" windowWidth="6756" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="37">
   <si>
     <t>file</t>
   </si>
@@ -471,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -1483,7 +1483,7 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F72" s="3">
-        <f t="shared" ref="F72:F117" si="1">E72-D72</f>
+        <f t="shared" ref="F72:F118" si="1">E72-D72</f>
         <v>0</v>
       </c>
       <c r="G72" s="3">
@@ -1721,450 +1721,471 @@
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B89" t="s">
+        <v>36</v>
+      </c>
+      <c r="C89" t="s">
+        <v>9</v>
+      </c>
+      <c r="D89" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E89" s="3">
+        <v>0.42499999999999999</v>
+      </c>
       <c r="F89" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G89" s="3">
-        <f>SUM(F87:F89)</f>
-        <v>3.1944444444444331E-2</v>
+        <v>8.3333333333333037E-3</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
+      <c r="D90" s="3">
+        <v>0.53125</v>
+      </c>
+      <c r="E90" s="3">
+        <v>0.54374999999999996</v>
+      </c>
+      <c r="F90" s="3">
+        <f t="shared" si="1"/>
+        <v>1.2499999999999956E-2</v>
+      </c>
+      <c r="G90" s="3">
+        <f>SUM(F87:F90)</f>
+        <v>5.277777777777759E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
         <v>26</v>
       </c>
-      <c r="B90" t="s">
-        <v>34</v>
-      </c>
-      <c r="C90" t="s">
-        <v>9</v>
-      </c>
-      <c r="D90" s="3">
+      <c r="B91" t="s">
+        <v>34</v>
+      </c>
+      <c r="C91" t="s">
+        <v>9</v>
+      </c>
+      <c r="D91" s="3">
         <v>0.52430555555555558</v>
       </c>
-      <c r="E90" s="3">
+      <c r="E91" s="3">
         <v>0.54305555555555551</v>
       </c>
-      <c r="F90" s="3">
+      <c r="F91" s="3">
         <f t="shared" si="1"/>
         <v>1.8749999999999933E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D91" s="3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D92" s="3">
         <v>0.54722222222222228</v>
       </c>
-      <c r="E91" s="3">
+      <c r="E92" s="3">
         <v>0.5541666666666667</v>
       </c>
-      <c r="F91" s="3">
+      <c r="F92" s="3">
         <f t="shared" si="1"/>
         <v>6.9444444444444198E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F92" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G92" s="3">
-        <f>SUM(F90:F92)</f>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F93" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G93" s="3">
+        <f>SUM(F91:F93)</f>
         <v>2.5694444444444353E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
         <v>27</v>
       </c>
-      <c r="B93" t="s">
-        <v>34</v>
-      </c>
-      <c r="C93" t="s">
-        <v>9</v>
-      </c>
-      <c r="D93" s="3">
+      <c r="B94" t="s">
+        <v>34</v>
+      </c>
+      <c r="C94" t="s">
+        <v>9</v>
+      </c>
+      <c r="D94" s="3">
         <v>0.46527777777777779</v>
       </c>
-      <c r="E93" s="3">
+      <c r="E94" s="3">
         <v>0.47569444444444442</v>
       </c>
-      <c r="F93" s="3">
+      <c r="F94" s="3">
         <f t="shared" si="1"/>
         <v>1.041666666666663E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D94" s="3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D95" s="3">
         <v>0.50694444444444442</v>
       </c>
-      <c r="E94" s="3">
+      <c r="E95" s="3">
         <v>0.51249999999999996</v>
       </c>
-      <c r="F94" s="3">
+      <c r="F95" s="3">
         <f t="shared" si="1"/>
         <v>5.5555555555555358E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F95" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G95" s="3">
-        <f>SUM(F93:F95)</f>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F96" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G96" s="3">
+        <f>SUM(F94:F96)</f>
         <v>1.5972222222222165E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>29</v>
       </c>
-      <c r="B96" t="s">
-        <v>34</v>
-      </c>
-      <c r="C96" t="s">
-        <v>9</v>
-      </c>
-      <c r="D96" s="3">
+      <c r="B97" t="s">
+        <v>34</v>
+      </c>
+      <c r="C97" t="s">
+        <v>9</v>
+      </c>
+      <c r="D97" s="3">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E96" s="3">
+      <c r="E97" s="3">
         <v>0.55763888888888891</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F97" s="3">
         <f t="shared" si="1"/>
         <v>1.5972222222222276E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B97" t="s">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
         <v>36</v>
       </c>
-      <c r="C97" t="s">
-        <v>9</v>
-      </c>
-      <c r="D97" s="3">
+      <c r="C98" t="s">
+        <v>9</v>
+      </c>
+      <c r="D98" s="3">
         <v>0.59513888888888888</v>
       </c>
-      <c r="E97" s="3">
+      <c r="E98" s="3">
         <v>0.61250000000000004</v>
       </c>
-      <c r="F97" s="3">
+      <c r="F98" s="3">
         <f t="shared" si="1"/>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F98" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G98" s="3">
-        <f>SUM(F96:F98)</f>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F99" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G99" s="3">
+        <f>SUM(F97:F99)</f>
         <v>3.3333333333333437E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
         <v>28</v>
       </c>
-      <c r="B99" t="s">
-        <v>34</v>
-      </c>
-      <c r="C99" t="s">
-        <v>9</v>
-      </c>
-      <c r="D99" s="3">
+      <c r="B100" t="s">
+        <v>34</v>
+      </c>
+      <c r="C100" t="s">
+        <v>9</v>
+      </c>
+      <c r="D100" s="3">
         <v>0.53472222222222221</v>
       </c>
-      <c r="E99" s="3">
+      <c r="E100" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="F99" s="3">
+      <c r="F100" s="3">
         <f t="shared" si="1"/>
         <v>3.819444444444442E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B100" t="s">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B101" t="s">
         <v>36</v>
       </c>
-      <c r="C100" t="s">
-        <v>9</v>
-      </c>
-      <c r="D100" s="3">
+      <c r="C101" t="s">
+        <v>9</v>
+      </c>
+      <c r="D101" s="3">
         <v>0.61597222222222225</v>
       </c>
-      <c r="E100" s="3">
+      <c r="E101" s="3">
         <v>0.62152777777777779</v>
       </c>
-      <c r="F100" s="3">
+      <c r="F101" s="3">
         <f t="shared" si="1"/>
         <v>5.5555555555555358E-3</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D101" s="3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D102" s="3">
         <v>0.57291666666666663</v>
       </c>
-      <c r="E101" s="3">
+      <c r="E102" s="3">
         <v>0.59097222222222223</v>
       </c>
-      <c r="F101" s="3">
+      <c r="F102" s="3">
         <f t="shared" si="1"/>
         <v>1.8055555555555602E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F102" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G102" s="3">
-        <f>SUM(F99:F102)</f>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F103" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G103" s="3">
+        <f>SUM(F100:F103)</f>
         <v>6.1805555555555558E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
         <v>30</v>
       </c>
-      <c r="B103" t="s">
-        <v>34</v>
-      </c>
-      <c r="C103" t="s">
-        <v>9</v>
-      </c>
-      <c r="D103" s="3">
+      <c r="B104" t="s">
+        <v>34</v>
+      </c>
+      <c r="C104" t="s">
+        <v>9</v>
+      </c>
+      <c r="D104" s="3">
         <v>0.54652777777777772</v>
       </c>
-      <c r="E103" s="3">
+      <c r="E104" s="3">
         <v>0.56736111111111109</v>
       </c>
-      <c r="F103" s="3">
+      <c r="F104" s="3">
         <f t="shared" si="1"/>
         <v>2.083333333333337E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B104" t="s">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B105" t="s">
         <v>36</v>
       </c>
-      <c r="C104" t="s">
-        <v>9</v>
-      </c>
-      <c r="D104" s="3">
+      <c r="C105" t="s">
+        <v>9</v>
+      </c>
+      <c r="D105" s="3">
         <v>0.59513888888888888</v>
       </c>
-      <c r="E104" s="3">
+      <c r="E105" s="3">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F104" s="3">
+      <c r="F105" s="3">
         <f t="shared" si="1"/>
         <v>9.0277777777777457E-3</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F105" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G105" s="3">
-        <f>SUM(F103:F105)</f>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F106" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G106" s="3">
+        <f>SUM(F104:F106)</f>
         <v>2.9861111111111116E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
         <v>31</v>
       </c>
-      <c r="B106" t="s">
-        <v>34</v>
-      </c>
-      <c r="C106" t="s">
-        <v>9</v>
-      </c>
-      <c r="D106" s="3">
+      <c r="B107" t="s">
+        <v>34</v>
+      </c>
+      <c r="C107" t="s">
+        <v>9</v>
+      </c>
+      <c r="D107" s="3">
         <v>0.78125</v>
       </c>
-      <c r="E106" s="3">
+      <c r="E107" s="3">
         <v>0.80555555555555558</v>
       </c>
-      <c r="F106" s="3">
+      <c r="F107" s="3">
         <f t="shared" si="1"/>
         <v>2.430555555555558E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B107" t="s">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B108" t="s">
         <v>36</v>
       </c>
-      <c r="C107" t="s">
-        <v>9</v>
-      </c>
-      <c r="D107" s="3">
+      <c r="C108" t="s">
+        <v>9</v>
+      </c>
+      <c r="D108" s="3">
         <v>0.5444444444444444</v>
       </c>
-      <c r="E107" s="3">
+      <c r="E108" s="3">
         <v>0.55555555555555558</v>
       </c>
-      <c r="F107" s="3">
+      <c r="F108" s="3">
         <f t="shared" si="1"/>
         <v>1.1111111111111183E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F108" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G108" s="3">
-        <f>SUM(F106:F107)</f>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F109" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G109" s="3">
+        <f>SUM(F107:F108)</f>
         <v>3.5416666666666763E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
         <v>32</v>
       </c>
-      <c r="B109" t="s">
-        <v>34</v>
-      </c>
-      <c r="C109" t="s">
-        <v>9</v>
-      </c>
-      <c r="D109" s="3">
+      <c r="B110" t="s">
+        <v>34</v>
+      </c>
+      <c r="C110" t="s">
+        <v>9</v>
+      </c>
+      <c r="D110" s="3">
         <v>0.8125</v>
       </c>
-      <c r="E109" s="3">
+      <c r="E110" s="3">
         <v>0.82986111111111116</v>
       </c>
-      <c r="F109" s="3">
+      <c r="F110" s="3">
         <f t="shared" si="1"/>
         <v>1.736111111111116E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B110" t="s">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B111" t="s">
         <v>36</v>
       </c>
-      <c r="C110" t="s">
-        <v>9</v>
-      </c>
-      <c r="D110" s="3">
+      <c r="C111" t="s">
+        <v>9</v>
+      </c>
+      <c r="D111" s="3">
         <v>0.65486111111111112</v>
       </c>
-      <c r="E110" s="3">
+      <c r="E111" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="F110" s="3">
+      <c r="F111" s="3">
         <f t="shared" si="1"/>
         <v>1.1805555555555514E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F111" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G111" s="3">
-        <f>SUM(F109:F111)</f>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F112" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G112" s="3">
+        <f>SUM(F110:F112)</f>
         <v>2.9166666666666674E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A112" t="s">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
         <v>33</v>
       </c>
-      <c r="B112" t="s">
-        <v>34</v>
-      </c>
-      <c r="C112" t="s">
-        <v>9</v>
-      </c>
-      <c r="D112" s="3">
+      <c r="B113" t="s">
+        <v>34</v>
+      </c>
+      <c r="C113" t="s">
+        <v>9</v>
+      </c>
+      <c r="D113" s="3">
         <v>0.59166666666666667</v>
       </c>
-      <c r="E112" s="3">
+      <c r="E113" s="3">
         <v>0.66666666666666663</v>
       </c>
-      <c r="F112" s="3">
+      <c r="F113" s="3">
         <f t="shared" si="1"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
-    <row r="113" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D113" s="3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D114" s="3">
         <v>0.78888888888888886</v>
       </c>
-      <c r="E113" s="3">
+      <c r="E114" s="3">
         <v>0.83680555555555558</v>
       </c>
-      <c r="F113" s="3">
+      <c r="F114" s="3">
         <f t="shared" si="1"/>
         <v>4.7916666666666718E-2</v>
       </c>
-      <c r="G113" s="3">
-        <f>SUM(F112:F113)</f>
+      <c r="G114" s="3">
+        <f>SUM(F113:F114)</f>
         <v>0.12291666666666667</v>
       </c>
     </row>
-    <row r="114" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="F114" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F115" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F116" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F117" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="F118" s="3"/>
-    </row>
-    <row r="119" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F118" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F119" s="3"/>
     </row>
-    <row r="120" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F120" s="3"/>
     </row>
-    <row r="121" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F121" s="3"/>
     </row>
-    <row r="122" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F122" s="3"/>
     </row>
-    <row r="123" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F123" s="3"/>
     </row>
-    <row r="124" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F124" s="3"/>
     </row>
-    <row r="125" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F125" s="3"/>
     </row>
-    <row r="126" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F126" s="3"/>
     </row>
-    <row r="127" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F127" s="3"/>
     </row>
-    <row r="128" spans="4:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F128" s="3"/>
     </row>
     <row r="129" spans="6:6" x14ac:dyDescent="0.3">
@@ -2184,6 +2205,9 @@
     </row>
     <row r="134" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F134" s="3"/>
+    </row>
+    <row r="135" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F135" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added discourse annotations for parcor
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B27D7DF-EC65-47B1-8A4F-F1B18EBB4659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D5C11C-FC73-4691-A2BC-E7A8638EAC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16380" yWindow="0" windowWidth="6756" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16932" yWindow="0" windowWidth="6204" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="37">
   <si>
     <t>file</t>
   </si>
@@ -1427,13 +1427,25 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" s="3">
+        <v>0.52847222222222223</v>
+      </c>
+      <c r="E68" s="3">
+        <v>0.5395833333333333</v>
+      </c>
       <c r="F68" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.1111111111111072E-2</v>
       </c>
       <c r="G68" s="3">
         <f>SUM(F65:F68)</f>
-        <v>4.2361111111111183E-2</v>
+        <v>5.3472222222222254E-2</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
@@ -1562,19 +1574,37 @@
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B78" t="s">
+        <v>36</v>
+      </c>
+      <c r="C78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D78" s="3">
+        <v>0.51875000000000004</v>
+      </c>
+      <c r="E78" s="3">
+        <v>0.52083333333333337</v>
+      </c>
       <c r="F78" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.0833333333333259E-3</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D79" s="3">
+        <v>0.49861111111111112</v>
+      </c>
+      <c r="E79" s="3">
+        <v>0.51527777777777772</v>
+      </c>
       <c r="F79" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.6666666666666607E-2</v>
       </c>
       <c r="G79" s="3">
         <f>SUM(F77:F79)</f>
-        <v>2.2222222222222254E-2</v>
+        <v>4.0972222222222188E-2</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
@@ -1831,13 +1861,25 @@
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B96" t="s">
+        <v>36</v>
+      </c>
+      <c r="C96" t="s">
+        <v>9</v>
+      </c>
+      <c r="D96" s="3">
+        <v>0.52013888888888893</v>
+      </c>
+      <c r="E96" s="3">
+        <v>0.52638888888888891</v>
+      </c>
       <c r="F96" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6.2499999999999778E-3</v>
       </c>
       <c r="G96" s="3">
         <f>SUM(F94:F96)</f>
-        <v>1.5972222222222165E-2</v>
+        <v>2.2222222222222143E-2</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added hypophora overview and discourse annotations
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2308B9-83DB-42B9-82A3-4CCE005BF61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60C5A7D-F07E-4279-AD23-82469D36C6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15588" yWindow="0" windowWidth="7548" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -2207,10 +2207,6 @@
         <f t="shared" si="1"/>
         <v>4.7916666666666718E-2</v>
       </c>
-      <c r="G114" s="3">
-        <f>SUM(F113:F114)</f>
-        <v>0.12291666666666667</v>
-      </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
@@ -2219,15 +2215,25 @@
       <c r="C115" t="s">
         <v>9</v>
       </c>
+      <c r="D115" s="3">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="E115" s="3">
+        <v>0.625</v>
+      </c>
       <c r="F115" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.513888888888884E-2</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F116" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
+      </c>
+      <c r="G116" s="3">
+        <f>SUM(F113:F116)</f>
+        <v>0.16805555555555551</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
updated discourse annotation teddy-744
</commit_message>
<xml_diff>
--- a/annotators/team/tg/de/cost_annotation_times.xlsx
+++ b/annotators/team/tg/de/cost_annotation_times.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\Git\AURIS\annotators\team\tg\de\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tabea\Desktop\AURIS\annotators\team\tg\de\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60C5A7D-F07E-4279-AD23-82469D36C6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62FD18F8-CC55-4A8F-AEBF-A74523FBC704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2227,13 +2227,19 @@
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D116" s="3">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="E116" s="3">
+        <v>0.59722222222222221</v>
+      </c>
       <c r="F116" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.430555555555558E-2</v>
       </c>
       <c r="G116" s="3">
         <f>SUM(F113:F116)</f>
-        <v>0.16805555555555551</v>
+        <v>0.19236111111111109</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>